<commit_message>
update xlx and format
</commit_message>
<xml_diff>
--- a/foo.xlsx
+++ b/foo.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{3CB7D34E-61B1-45D5-A9DB-ECE44F5F9BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2CA593FC-C934-4EE9-A60C-530B780172E7}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{2CA593FC-C934-4EE9-A60C-530B780172E7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1142,38 +1142,11 @@
     <xf numFmtId="3" fontId="3" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="43" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1194,8 +1167,35 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="43" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="9">
@@ -1543,16 +1543,16 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A1" s="67" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
+      <c r="A1" s="58" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -1572,8 +1572,8 @@
       <c r="W1" s="1"/>
     </row>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="69"/>
-      <c r="B2" s="69"/>
+      <c r="A2" s="60"/>
+      <c r="B2" s="60"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
@@ -1597,35 +1597,35 @@
       <c r="W2" s="1"/>
     </row>
     <row r="3" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="70" t="s">
+      <c r="A3" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="72" t="s">
+      <c r="B3" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="56" t="s">
+      <c r="C3" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="58"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="66"/>
+      <c r="F3" s="66"/>
+      <c r="G3" s="66"/>
+      <c r="H3" s="67"/>
       <c r="I3" s="1"/>
-      <c r="J3" s="70" t="s">
+      <c r="J3" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="72" t="s">
+      <c r="K3" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="L3" s="56" t="s">
+      <c r="L3" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="M3" s="57"/>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="58"/>
+      <c r="M3" s="66"/>
+      <c r="N3" s="66"/>
+      <c r="O3" s="66"/>
+      <c r="P3" s="66"/>
+      <c r="Q3" s="67"/>
       <c r="R3" s="1"/>
       <c r="S3" s="1"/>
       <c r="T3" s="1"/>
@@ -1634,35 +1634,35 @@
       <c r="W3" s="1"/>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A4" s="71"/>
-      <c r="B4" s="73"/>
-      <c r="C4" s="59">
+      <c r="A4" s="62"/>
+      <c r="B4" s="64"/>
+      <c r="C4" s="73">
         <v>2025</v>
       </c>
-      <c r="D4" s="60"/>
-      <c r="E4" s="59">
+      <c r="D4" s="74"/>
+      <c r="E4" s="73">
         <v>2026</v>
       </c>
-      <c r="F4" s="60"/>
-      <c r="G4" s="59" t="s">
+      <c r="F4" s="74"/>
+      <c r="G4" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="60"/>
+      <c r="H4" s="74"/>
       <c r="I4" s="1"/>
-      <c r="J4" s="71"/>
-      <c r="K4" s="73"/>
-      <c r="L4" s="59">
+      <c r="J4" s="62"/>
+      <c r="K4" s="64"/>
+      <c r="L4" s="73">
         <v>2025</v>
       </c>
-      <c r="M4" s="60"/>
-      <c r="N4" s="59">
+      <c r="M4" s="74"/>
+      <c r="N4" s="73">
         <v>2026</v>
       </c>
-      <c r="O4" s="60"/>
-      <c r="P4" s="59" t="s">
+      <c r="O4" s="74"/>
+      <c r="P4" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="Q4" s="60"/>
+      <c r="Q4" s="74"/>
       <c r="R4" s="1"/>
       <c r="S4" s="1"/>
       <c r="T4" s="1"/>
@@ -1671,8 +1671,8 @@
       <c r="W4" s="1"/>
     </row>
     <row r="5" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="71"/>
-      <c r="B5" s="73"/>
+      <c r="A5" s="62"/>
+      <c r="B5" s="64"/>
       <c r="C5" s="41" t="s">
         <v>6</v>
       </c>
@@ -1692,8 +1692,8 @@
         <v>9</v>
       </c>
       <c r="I5" s="1"/>
-      <c r="J5" s="71"/>
-      <c r="K5" s="73"/>
+      <c r="J5" s="62"/>
+      <c r="K5" s="64"/>
       <c r="L5" s="41" t="s">
         <v>6</v>
       </c>
@@ -2102,7 +2102,7 @@
       </c>
     </row>
     <row r="12" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="62">
+      <c r="A12" s="68">
         <v>6</v>
       </c>
       <c r="B12" s="34" t="s">
@@ -2127,7 +2127,7 @@
         <v>8.1027711604049806</v>
       </c>
       <c r="I12" s="4"/>
-      <c r="J12" s="62">
+      <c r="J12" s="68">
         <v>6</v>
       </c>
       <c r="K12" s="34" t="s">
@@ -2167,7 +2167,7 @@
       </c>
     </row>
     <row r="13" spans="1:23" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="63"/>
+      <c r="A13" s="69"/>
       <c r="B13" s="35" t="s">
         <v>16</v>
       </c>
@@ -2190,7 +2190,7 @@
         <v>7.6388930682784535</v>
       </c>
       <c r="I13" s="4"/>
-      <c r="J13" s="63"/>
+      <c r="J13" s="69"/>
       <c r="K13" s="35" t="s">
         <v>16</v>
       </c>
@@ -2228,7 +2228,7 @@
       </c>
     </row>
     <row r="14" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="62">
+      <c r="A14" s="68">
         <v>7</v>
       </c>
       <c r="B14" s="32" t="s">
@@ -2253,7 +2253,7 @@
         <v>8.7531970882529535</v>
       </c>
       <c r="I14" s="4"/>
-      <c r="J14" s="62">
+      <c r="J14" s="68">
         <v>7</v>
       </c>
       <c r="K14" s="32" t="s">
@@ -2293,7 +2293,7 @@
       </c>
     </row>
     <row r="15" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="64"/>
+      <c r="A15" s="70"/>
       <c r="B15" s="36" t="s">
         <v>18</v>
       </c>
@@ -2316,7 +2316,7 @@
         <v>9.9400475446276921</v>
       </c>
       <c r="I15" s="4"/>
-      <c r="J15" s="64"/>
+      <c r="J15" s="70"/>
       <c r="K15" s="36" t="s">
         <v>18</v>
       </c>
@@ -2354,10 +2354,10 @@
       </c>
     </row>
     <row r="16" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="65" t="s">
+      <c r="A16" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="66"/>
+      <c r="B16" s="72"/>
       <c r="C16" s="17">
         <v>2983.9677000000001</v>
       </c>
@@ -2377,10 +2377,10 @@
         <v>7.9465877552996211</v>
       </c>
       <c r="I16" s="4"/>
-      <c r="J16" s="65" t="s">
+      <c r="J16" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="K16" s="66"/>
+      <c r="K16" s="72"/>
       <c r="L16" s="17">
         <v>2983.9677000000001</v>
       </c>
@@ -2480,16 +2480,16 @@
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A18" s="61" t="s">
+      <c r="A18" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="61"/>
-      <c r="C18" s="61"/>
-      <c r="D18" s="61"/>
-      <c r="E18" s="61"/>
-      <c r="F18" s="61"/>
-      <c r="G18" s="61"/>
-      <c r="H18" s="61"/>
+      <c r="B18" s="56"/>
+      <c r="C18" s="56"/>
+      <c r="D18" s="56"/>
+      <c r="E18" s="56"/>
+      <c r="F18" s="56"/>
+      <c r="G18" s="56"/>
+      <c r="H18" s="56"/>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
@@ -2534,16 +2534,16 @@
       <c r="W19" s="1"/>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A20" s="67" t="s">
+      <c r="A20" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="68"/>
-      <c r="C20" s="68"/>
-      <c r="D20" s="68"/>
-      <c r="E20" s="68"/>
-      <c r="F20" s="68"/>
-      <c r="G20" s="68"/>
-      <c r="H20" s="68"/>
+      <c r="B20" s="59"/>
+      <c r="C20" s="59"/>
+      <c r="D20" s="59"/>
+      <c r="E20" s="59"/>
+      <c r="F20" s="59"/>
+      <c r="G20" s="59"/>
+      <c r="H20" s="59"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
@@ -2563,8 +2563,8 @@
       <c r="W20" s="1"/>
     </row>
     <row r="21" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="69"/>
-      <c r="B21" s="69"/>
+      <c r="A21" s="60"/>
+      <c r="B21" s="60"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
@@ -2588,35 +2588,35 @@
       <c r="W21" s="1"/>
     </row>
     <row r="22" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="70" t="s">
+      <c r="A22" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="B22" s="72" t="s">
+      <c r="B22" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="C22" s="56" t="s">
+      <c r="C22" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="D22" s="57"/>
-      <c r="E22" s="57"/>
-      <c r="F22" s="57"/>
-      <c r="G22" s="57"/>
-      <c r="H22" s="58"/>
+      <c r="D22" s="66"/>
+      <c r="E22" s="66"/>
+      <c r="F22" s="66"/>
+      <c r="G22" s="66"/>
+      <c r="H22" s="67"/>
       <c r="I22" s="1"/>
-      <c r="J22" s="70" t="s">
+      <c r="J22" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="K22" s="72" t="s">
+      <c r="K22" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="L22" s="56" t="s">
+      <c r="L22" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="M22" s="57"/>
-      <c r="N22" s="57"/>
-      <c r="O22" s="57"/>
-      <c r="P22" s="57"/>
-      <c r="Q22" s="58"/>
+      <c r="M22" s="66"/>
+      <c r="N22" s="66"/>
+      <c r="O22" s="66"/>
+      <c r="P22" s="66"/>
+      <c r="Q22" s="67"/>
       <c r="R22" s="1"/>
       <c r="S22" s="1"/>
       <c r="T22" s="1"/>
@@ -2625,35 +2625,35 @@
       <c r="W22" s="1"/>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A23" s="71"/>
-      <c r="B23" s="73"/>
-      <c r="C23" s="59">
+      <c r="A23" s="62"/>
+      <c r="B23" s="64"/>
+      <c r="C23" s="73">
         <v>2025</v>
       </c>
-      <c r="D23" s="60"/>
-      <c r="E23" s="59">
+      <c r="D23" s="74"/>
+      <c r="E23" s="73">
         <v>2026</v>
       </c>
-      <c r="F23" s="60"/>
-      <c r="G23" s="59" t="s">
+      <c r="F23" s="74"/>
+      <c r="G23" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="H23" s="60"/>
+      <c r="H23" s="74"/>
       <c r="I23" s="1"/>
-      <c r="J23" s="71"/>
-      <c r="K23" s="73"/>
-      <c r="L23" s="59">
+      <c r="J23" s="62"/>
+      <c r="K23" s="64"/>
+      <c r="L23" s="73">
         <v>2025</v>
       </c>
-      <c r="M23" s="60"/>
-      <c r="N23" s="59">
+      <c r="M23" s="74"/>
+      <c r="N23" s="73">
         <v>2026</v>
       </c>
-      <c r="O23" s="60"/>
-      <c r="P23" s="59" t="s">
+      <c r="O23" s="74"/>
+      <c r="P23" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="Q23" s="60"/>
+      <c r="Q23" s="74"/>
       <c r="R23" s="1"/>
       <c r="S23" s="1"/>
       <c r="T23" s="1"/>
@@ -2662,8 +2662,8 @@
       <c r="W23" s="1"/>
     </row>
     <row r="24" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="71"/>
-      <c r="B24" s="73"/>
+      <c r="A24" s="62"/>
+      <c r="B24" s="64"/>
       <c r="C24" s="41" t="s">
         <v>23</v>
       </c>
@@ -2683,8 +2683,8 @@
         <v>9</v>
       </c>
       <c r="I24" s="1"/>
-      <c r="J24" s="71"/>
-      <c r="K24" s="73"/>
+      <c r="J24" s="62"/>
+      <c r="K24" s="64"/>
       <c r="L24" s="41" t="s">
         <v>23</v>
       </c>
@@ -3093,7 +3093,7 @@
       </c>
     </row>
     <row r="31" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="62">
+      <c r="A31" s="68">
         <v>6</v>
       </c>
       <c r="B31" s="34" t="s">
@@ -3118,7 +3118,7 @@
         <v>8.7465726084095721</v>
       </c>
       <c r="I31" s="4"/>
-      <c r="J31" s="62">
+      <c r="J31" s="68">
         <v>6</v>
       </c>
       <c r="K31" s="34" t="s">
@@ -3158,7 +3158,7 @@
       </c>
     </row>
     <row r="32" spans="1:23" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="63"/>
+      <c r="A32" s="69"/>
       <c r="B32" s="35" t="s">
         <v>16</v>
       </c>
@@ -3181,7 +3181,7 @@
         <v>8.2270982911297796</v>
       </c>
       <c r="I32" s="4"/>
-      <c r="J32" s="63"/>
+      <c r="J32" s="69"/>
       <c r="K32" s="35" t="s">
         <v>16</v>
       </c>
@@ -3219,7 +3219,7 @@
       </c>
     </row>
     <row r="33" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="62">
+      <c r="A33" s="68">
         <v>7</v>
       </c>
       <c r="B33" s="32" t="s">
@@ -3244,7 +3244,7 @@
         <v>9.6491696800585807</v>
       </c>
       <c r="I33" s="4"/>
-      <c r="J33" s="62">
+      <c r="J33" s="68">
         <v>7</v>
       </c>
       <c r="K33" s="32" t="s">
@@ -3284,7 +3284,7 @@
       </c>
     </row>
     <row r="34" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="64"/>
+      <c r="A34" s="70"/>
       <c r="B34" s="36" t="s">
         <v>18</v>
       </c>
@@ -3307,7 +3307,7 @@
         <v>10.799000367826759</v>
       </c>
       <c r="I34" s="4"/>
-      <c r="J34" s="64"/>
+      <c r="J34" s="70"/>
       <c r="K34" s="36" t="s">
         <v>18</v>
       </c>
@@ -3345,10 +3345,10 @@
       </c>
     </row>
     <row r="35" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="65" t="s">
+      <c r="A35" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="B35" s="66"/>
+      <c r="B35" s="72"/>
       <c r="C35" s="17">
         <v>3194.1713999999997</v>
       </c>
@@ -3368,10 +3368,10 @@
         <v>8.6919639725101838</v>
       </c>
       <c r="I35" s="4"/>
-      <c r="J35" s="65" t="s">
+      <c r="J35" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="K35" s="66"/>
+      <c r="K35" s="72"/>
       <c r="L35" s="17">
         <v>3194.1714000000002</v>
       </c>
@@ -3471,16 +3471,16 @@
       </c>
     </row>
     <row r="37" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A37" s="61" t="s">
+      <c r="A37" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="B37" s="61"/>
-      <c r="C37" s="61"/>
-      <c r="D37" s="61"/>
-      <c r="E37" s="61"/>
-      <c r="F37" s="61"/>
-      <c r="G37" s="61"/>
-      <c r="H37" s="61"/>
+      <c r="B37" s="56"/>
+      <c r="C37" s="56"/>
+      <c r="D37" s="56"/>
+      <c r="E37" s="56"/>
+      <c r="F37" s="56"/>
+      <c r="G37" s="56"/>
+      <c r="H37" s="56"/>
       <c r="I37" s="1"/>
       <c r="J37" s="1"/>
       <c r="K37" s="1"/>
@@ -3498,16 +3498,16 @@
       <c r="W37" s="1"/>
     </row>
     <row r="39" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A39" s="67" t="s">
+      <c r="A39" s="58" t="s">
         <v>25</v>
       </c>
-      <c r="B39" s="68"/>
-      <c r="C39" s="68"/>
-      <c r="D39" s="68"/>
-      <c r="E39" s="68"/>
-      <c r="F39" s="68"/>
-      <c r="G39" s="68"/>
-      <c r="H39" s="68"/>
+      <c r="B39" s="59"/>
+      <c r="C39" s="59"/>
+      <c r="D39" s="59"/>
+      <c r="E39" s="59"/>
+      <c r="F39" s="59"/>
+      <c r="G39" s="59"/>
+      <c r="H39" s="59"/>
       <c r="I39" s="1"/>
       <c r="J39" s="1"/>
       <c r="K39" s="1"/>
@@ -3527,8 +3527,8 @@
       <c r="W39" s="1"/>
     </row>
     <row r="40" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="69"/>
-      <c r="B40" s="69"/>
+      <c r="A40" s="60"/>
+      <c r="B40" s="60"/>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
       <c r="E40" s="2"/>
@@ -3552,35 +3552,35 @@
       <c r="W40" s="1"/>
     </row>
     <row r="41" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="70" t="s">
+      <c r="A41" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="B41" s="72" t="s">
+      <c r="B41" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="C41" s="56" t="s">
+      <c r="C41" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="D41" s="57"/>
-      <c r="E41" s="57"/>
-      <c r="F41" s="57"/>
-      <c r="G41" s="57"/>
-      <c r="H41" s="58"/>
+      <c r="D41" s="66"/>
+      <c r="E41" s="66"/>
+      <c r="F41" s="66"/>
+      <c r="G41" s="66"/>
+      <c r="H41" s="67"/>
       <c r="I41" s="1"/>
-      <c r="J41" s="70" t="s">
+      <c r="J41" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="K41" s="72" t="s">
+      <c r="K41" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="L41" s="56" t="s">
+      <c r="L41" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="M41" s="57"/>
-      <c r="N41" s="57"/>
-      <c r="O41" s="57"/>
-      <c r="P41" s="57"/>
-      <c r="Q41" s="58"/>
+      <c r="M41" s="66"/>
+      <c r="N41" s="66"/>
+      <c r="O41" s="66"/>
+      <c r="P41" s="66"/>
+      <c r="Q41" s="67"/>
       <c r="R41" s="1"/>
       <c r="S41" s="1"/>
       <c r="T41" s="1"/>
@@ -3589,35 +3589,35 @@
       <c r="W41" s="1"/>
     </row>
     <row r="42" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A42" s="71"/>
-      <c r="B42" s="73"/>
-      <c r="C42" s="59">
+      <c r="A42" s="62"/>
+      <c r="B42" s="64"/>
+      <c r="C42" s="73">
         <v>2025</v>
       </c>
-      <c r="D42" s="60"/>
-      <c r="E42" s="59">
+      <c r="D42" s="74"/>
+      <c r="E42" s="73">
         <v>2026</v>
       </c>
-      <c r="F42" s="60"/>
-      <c r="G42" s="59" t="s">
+      <c r="F42" s="74"/>
+      <c r="G42" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="H42" s="60"/>
+      <c r="H42" s="74"/>
       <c r="I42" s="1"/>
-      <c r="J42" s="71"/>
-      <c r="K42" s="73"/>
-      <c r="L42" s="59">
+      <c r="J42" s="62"/>
+      <c r="K42" s="64"/>
+      <c r="L42" s="73">
         <v>2025</v>
       </c>
-      <c r="M42" s="60"/>
-      <c r="N42" s="59">
+      <c r="M42" s="74"/>
+      <c r="N42" s="73">
         <v>2026</v>
       </c>
-      <c r="O42" s="60"/>
-      <c r="P42" s="59" t="s">
+      <c r="O42" s="74"/>
+      <c r="P42" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="Q42" s="60"/>
+      <c r="Q42" s="74"/>
       <c r="R42" s="1"/>
       <c r="S42" s="1"/>
       <c r="T42" s="1"/>
@@ -3626,8 +3626,8 @@
       <c r="W42" s="1"/>
     </row>
     <row r="43" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="71"/>
-      <c r="B43" s="73"/>
+      <c r="A43" s="62"/>
+      <c r="B43" s="64"/>
       <c r="C43" s="41" t="s">
         <v>26</v>
       </c>
@@ -3647,8 +3647,8 @@
         <v>9</v>
       </c>
       <c r="I43" s="1"/>
-      <c r="J43" s="71"/>
-      <c r="K43" s="73"/>
+      <c r="J43" s="62"/>
+      <c r="K43" s="64"/>
       <c r="L43" s="41" t="s">
         <v>26</v>
       </c>
@@ -4057,7 +4057,7 @@
       </c>
     </row>
     <row r="50" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="62">
+      <c r="A50" s="68">
         <v>6</v>
       </c>
       <c r="B50" s="34" t="s">
@@ -4082,7 +4082,7 @@
         <v>9.6793823389794778</v>
       </c>
       <c r="I50" s="4"/>
-      <c r="J50" s="62">
+      <c r="J50" s="68">
         <v>6</v>
       </c>
       <c r="K50" s="34" t="s">
@@ -4122,7 +4122,7 @@
       </c>
     </row>
     <row r="51" spans="1:23" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="63"/>
+      <c r="A51" s="69"/>
       <c r="B51" s="35" t="s">
         <v>16</v>
       </c>
@@ -4145,7 +4145,7 @@
         <v>9.0731625896035553</v>
       </c>
       <c r="I51" s="4"/>
-      <c r="J51" s="63"/>
+      <c r="J51" s="69"/>
       <c r="K51" s="35" t="s">
         <v>16</v>
       </c>
@@ -4183,7 +4183,7 @@
       </c>
     </row>
     <row r="52" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="62">
+      <c r="A52" s="68">
         <v>7</v>
       </c>
       <c r="B52" s="32" t="s">
@@ -4208,7 +4208,7 @@
         <v>10.763472145117159</v>
       </c>
       <c r="I52" s="4"/>
-      <c r="J52" s="62">
+      <c r="J52" s="68">
         <v>7</v>
       </c>
       <c r="K52" s="32" t="s">
@@ -4248,7 +4248,7 @@
       </c>
     </row>
     <row r="53" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="64"/>
+      <c r="A53" s="70"/>
       <c r="B53" s="36" t="s">
         <v>18</v>
       </c>
@@ -4271,7 +4271,7 @@
         <v>12.019745543607423</v>
       </c>
       <c r="I53" s="4"/>
-      <c r="J53" s="64"/>
+      <c r="J53" s="70"/>
       <c r="K53" s="36" t="s">
         <v>18</v>
       </c>
@@ -4309,10 +4309,10 @@
       </c>
     </row>
     <row r="54" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="65" t="s">
+      <c r="A54" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="B54" s="66"/>
+      <c r="B54" s="72"/>
       <c r="C54" s="17">
         <v>3122.7218999999996</v>
       </c>
@@ -4332,10 +4332,10 @@
         <v>9.6620946407194186</v>
       </c>
       <c r="I54" s="4"/>
-      <c r="J54" s="65" t="s">
+      <c r="J54" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="K54" s="66"/>
+      <c r="K54" s="72"/>
       <c r="L54" s="17">
         <v>3122.7219</v>
       </c>
@@ -4435,16 +4435,16 @@
       </c>
     </row>
     <row r="56" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A56" s="61" t="s">
+      <c r="A56" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="B56" s="61"/>
-      <c r="C56" s="61"/>
-      <c r="D56" s="61"/>
-      <c r="E56" s="61"/>
-      <c r="F56" s="61"/>
-      <c r="G56" s="61"/>
-      <c r="H56" s="61"/>
+      <c r="B56" s="56"/>
+      <c r="C56" s="56"/>
+      <c r="D56" s="56"/>
+      <c r="E56" s="56"/>
+      <c r="F56" s="56"/>
+      <c r="G56" s="56"/>
+      <c r="H56" s="56"/>
       <c r="I56" s="1"/>
       <c r="J56" s="1"/>
       <c r="K56" s="1"/>
@@ -4462,16 +4462,16 @@
       <c r="W56" s="1"/>
     </row>
     <row r="58" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A58" s="67" t="s">
+      <c r="A58" s="58" t="s">
         <v>28</v>
       </c>
-      <c r="B58" s="68"/>
-      <c r="C58" s="68"/>
-      <c r="D58" s="68"/>
-      <c r="E58" s="68"/>
-      <c r="F58" s="68"/>
-      <c r="G58" s="68"/>
-      <c r="H58" s="68"/>
+      <c r="B58" s="59"/>
+      <c r="C58" s="59"/>
+      <c r="D58" s="59"/>
+      <c r="E58" s="59"/>
+      <c r="F58" s="59"/>
+      <c r="G58" s="59"/>
+      <c r="H58" s="59"/>
       <c r="I58" s="1"/>
       <c r="J58" s="1"/>
       <c r="K58" s="1"/>
@@ -4491,8 +4491,8 @@
       <c r="W58" s="1"/>
     </row>
     <row r="59" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="69"/>
-      <c r="B59" s="69"/>
+      <c r="A59" s="60"/>
+      <c r="B59" s="60"/>
       <c r="C59" s="2"/>
       <c r="D59" s="2"/>
       <c r="E59" s="2"/>
@@ -4516,35 +4516,35 @@
       <c r="W59" s="1"/>
     </row>
     <row r="60" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="70" t="s">
+      <c r="A60" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="B60" s="72" t="s">
+      <c r="B60" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="C60" s="56" t="s">
+      <c r="C60" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="D60" s="57"/>
-      <c r="E60" s="57"/>
-      <c r="F60" s="57"/>
-      <c r="G60" s="57"/>
-      <c r="H60" s="58"/>
+      <c r="D60" s="66"/>
+      <c r="E60" s="66"/>
+      <c r="F60" s="66"/>
+      <c r="G60" s="66"/>
+      <c r="H60" s="67"/>
       <c r="I60" s="1"/>
-      <c r="J60" s="70" t="s">
+      <c r="J60" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="K60" s="72" t="s">
+      <c r="K60" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="L60" s="56" t="s">
+      <c r="L60" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="M60" s="57"/>
-      <c r="N60" s="57"/>
-      <c r="O60" s="57"/>
-      <c r="P60" s="57"/>
-      <c r="Q60" s="58"/>
+      <c r="M60" s="66"/>
+      <c r="N60" s="66"/>
+      <c r="O60" s="66"/>
+      <c r="P60" s="66"/>
+      <c r="Q60" s="67"/>
       <c r="R60" s="1"/>
       <c r="S60" s="1"/>
       <c r="T60" s="1"/>
@@ -4553,35 +4553,35 @@
       <c r="W60" s="1"/>
     </row>
     <row r="61" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A61" s="71"/>
-      <c r="B61" s="73"/>
-      <c r="C61" s="59">
+      <c r="A61" s="62"/>
+      <c r="B61" s="64"/>
+      <c r="C61" s="73">
         <v>2025</v>
       </c>
-      <c r="D61" s="60"/>
-      <c r="E61" s="59">
+      <c r="D61" s="74"/>
+      <c r="E61" s="73">
         <v>2026</v>
       </c>
-      <c r="F61" s="60"/>
-      <c r="G61" s="59" t="s">
+      <c r="F61" s="74"/>
+      <c r="G61" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="H61" s="60"/>
+      <c r="H61" s="74"/>
       <c r="I61" s="1"/>
-      <c r="J61" s="71"/>
-      <c r="K61" s="73"/>
-      <c r="L61" s="59">
+      <c r="J61" s="62"/>
+      <c r="K61" s="64"/>
+      <c r="L61" s="73">
         <v>2025</v>
       </c>
-      <c r="M61" s="60"/>
-      <c r="N61" s="59">
+      <c r="M61" s="74"/>
+      <c r="N61" s="73">
         <v>2026</v>
       </c>
-      <c r="O61" s="60"/>
-      <c r="P61" s="59" t="s">
+      <c r="O61" s="74"/>
+      <c r="P61" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="Q61" s="60"/>
+      <c r="Q61" s="74"/>
       <c r="R61" s="1"/>
       <c r="S61" s="1"/>
       <c r="T61" s="1"/>
@@ -4590,8 +4590,8 @@
       <c r="W61" s="1"/>
     </row>
     <row r="62" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="71"/>
-      <c r="B62" s="73"/>
+      <c r="A62" s="62"/>
+      <c r="B62" s="64"/>
       <c r="C62" s="41" t="s">
         <v>29</v>
       </c>
@@ -4611,8 +4611,8 @@
         <v>9</v>
       </c>
       <c r="I62" s="1"/>
-      <c r="J62" s="71"/>
-      <c r="K62" s="73"/>
+      <c r="J62" s="62"/>
+      <c r="K62" s="64"/>
       <c r="L62" s="41" t="s">
         <v>29</v>
       </c>
@@ -5021,7 +5021,7 @@
       </c>
     </row>
     <row r="69" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="62">
+      <c r="A69" s="68">
         <v>6</v>
       </c>
       <c r="B69" s="34" t="s">
@@ -5046,7 +5046,7 @@
         <v>10.914496860390758</v>
       </c>
       <c r="I69" s="4"/>
-      <c r="J69" s="62">
+      <c r="J69" s="68">
         <v>6</v>
       </c>
       <c r="K69" s="34" t="s">
@@ -5086,7 +5086,7 @@
       </c>
     </row>
     <row r="70" spans="1:23" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="63"/>
+      <c r="A70" s="69"/>
       <c r="B70" s="35" t="s">
         <v>16</v>
       </c>
@@ -5111,7 +5111,7 @@
       <c r="I70" s="4">
         <v>-8895.8549999999996</v>
       </c>
-      <c r="J70" s="63"/>
+      <c r="J70" s="69"/>
       <c r="K70" s="35" t="s">
         <v>16</v>
       </c>
@@ -5149,7 +5149,7 @@
       </c>
     </row>
     <row r="71" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="62">
+      <c r="A71" s="68">
         <v>7</v>
       </c>
       <c r="B71" s="32" t="s">
@@ -5174,7 +5174,7 @@
         <v>12.168391481593714</v>
       </c>
       <c r="I71" s="4"/>
-      <c r="J71" s="62">
+      <c r="J71" s="68">
         <v>7</v>
       </c>
       <c r="K71" s="32" t="s">
@@ -5214,7 +5214,7 @@
       </c>
     </row>
     <row r="72" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="64"/>
+      <c r="A72" s="70"/>
       <c r="B72" s="36" t="s">
         <v>18</v>
       </c>
@@ -5239,7 +5239,7 @@
       <c r="I72" s="4">
         <v>-3973.3657999999996</v>
       </c>
-      <c r="J72" s="64"/>
+      <c r="J72" s="70"/>
       <c r="K72" s="36" t="s">
         <v>18</v>
       </c>
@@ -5277,10 +5277,10 @@
       </c>
     </row>
     <row r="73" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="65" t="s">
+      <c r="A73" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="B73" s="66"/>
+      <c r="B73" s="72"/>
       <c r="C73" s="17">
         <v>2948.3727000000003</v>
       </c>
@@ -5300,10 +5300,10 @@
         <v>10.845510569415543</v>
       </c>
       <c r="I73" s="4"/>
-      <c r="J73" s="65" t="s">
+      <c r="J73" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="K73" s="66"/>
+      <c r="K73" s="72"/>
       <c r="L73" s="46">
         <v>2948.3727000000008</v>
       </c>
@@ -5405,16 +5405,16 @@
       </c>
     </row>
     <row r="75" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A75" s="61" t="s">
+      <c r="A75" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="B75" s="61"/>
-      <c r="C75" s="61"/>
-      <c r="D75" s="61"/>
-      <c r="E75" s="61"/>
-      <c r="F75" s="61"/>
-      <c r="G75" s="61"/>
-      <c r="H75" s="61"/>
+      <c r="B75" s="56"/>
+      <c r="C75" s="56"/>
+      <c r="D75" s="56"/>
+      <c r="E75" s="56"/>
+      <c r="F75" s="56"/>
+      <c r="G75" s="56"/>
+      <c r="H75" s="56"/>
       <c r="I75" s="1"/>
       <c r="J75" s="1"/>
       <c r="K75" s="1"/>
@@ -5432,16 +5432,16 @@
       <c r="W75" s="1"/>
     </row>
     <row r="77" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A77" s="67" t="s">
+      <c r="A77" s="58" t="s">
         <v>31</v>
       </c>
-      <c r="B77" s="68"/>
-      <c r="C77" s="68"/>
-      <c r="D77" s="68"/>
-      <c r="E77" s="68"/>
-      <c r="F77" s="68"/>
-      <c r="G77" s="68"/>
-      <c r="H77" s="68"/>
+      <c r="B77" s="59"/>
+      <c r="C77" s="59"/>
+      <c r="D77" s="59"/>
+      <c r="E77" s="59"/>
+      <c r="F77" s="59"/>
+      <c r="G77" s="59"/>
+      <c r="H77" s="59"/>
       <c r="I77" s="1"/>
       <c r="J77" s="1"/>
       <c r="K77" s="1"/>
@@ -5461,8 +5461,8 @@
       <c r="W77" s="1"/>
     </row>
     <row r="78" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="69"/>
-      <c r="B78" s="69"/>
+      <c r="A78" s="60"/>
+      <c r="B78" s="60"/>
       <c r="C78" s="2"/>
       <c r="D78" s="2"/>
       <c r="E78" s="2"/>
@@ -5486,35 +5486,35 @@
       <c r="W78" s="1"/>
     </row>
     <row r="79" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="70" t="s">
+      <c r="A79" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="B79" s="72" t="s">
+      <c r="B79" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="C79" s="56" t="s">
+      <c r="C79" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="D79" s="57"/>
-      <c r="E79" s="57"/>
-      <c r="F79" s="57"/>
-      <c r="G79" s="57"/>
-      <c r="H79" s="58"/>
+      <c r="D79" s="66"/>
+      <c r="E79" s="66"/>
+      <c r="F79" s="66"/>
+      <c r="G79" s="66"/>
+      <c r="H79" s="67"/>
       <c r="I79" s="1"/>
-      <c r="J79" s="70" t="s">
+      <c r="J79" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="K79" s="72" t="s">
+      <c r="K79" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="L79" s="56" t="s">
+      <c r="L79" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="M79" s="57"/>
-      <c r="N79" s="57"/>
-      <c r="O79" s="57"/>
-      <c r="P79" s="57"/>
-      <c r="Q79" s="58"/>
+      <c r="M79" s="66"/>
+      <c r="N79" s="66"/>
+      <c r="O79" s="66"/>
+      <c r="P79" s="66"/>
+      <c r="Q79" s="67"/>
       <c r="R79" s="1"/>
       <c r="S79" s="1"/>
       <c r="T79" s="1"/>
@@ -5523,35 +5523,35 @@
       <c r="W79" s="1"/>
     </row>
     <row r="80" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A80" s="71"/>
-      <c r="B80" s="73"/>
-      <c r="C80" s="59">
+      <c r="A80" s="62"/>
+      <c r="B80" s="64"/>
+      <c r="C80" s="73">
         <v>2025</v>
       </c>
-      <c r="D80" s="60"/>
-      <c r="E80" s="59">
+      <c r="D80" s="74"/>
+      <c r="E80" s="73">
         <v>2026</v>
       </c>
-      <c r="F80" s="60"/>
-      <c r="G80" s="59" t="s">
+      <c r="F80" s="74"/>
+      <c r="G80" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="H80" s="60"/>
+      <c r="H80" s="74"/>
       <c r="I80" s="1"/>
-      <c r="J80" s="71"/>
-      <c r="K80" s="73"/>
-      <c r="L80" s="59">
+      <c r="J80" s="62"/>
+      <c r="K80" s="64"/>
+      <c r="L80" s="73">
         <v>2025</v>
       </c>
-      <c r="M80" s="60"/>
-      <c r="N80" s="59">
+      <c r="M80" s="74"/>
+      <c r="N80" s="73">
         <v>2026</v>
       </c>
-      <c r="O80" s="60"/>
-      <c r="P80" s="59" t="s">
+      <c r="O80" s="74"/>
+      <c r="P80" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="Q80" s="60"/>
+      <c r="Q80" s="74"/>
       <c r="R80" s="1"/>
       <c r="S80" s="1"/>
       <c r="T80" s="1"/>
@@ -5560,8 +5560,8 @@
       <c r="W80" s="1"/>
     </row>
     <row r="81" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="71"/>
-      <c r="B81" s="73"/>
+      <c r="A81" s="62"/>
+      <c r="B81" s="64"/>
       <c r="C81" s="41" t="s">
         <v>32</v>
       </c>
@@ -5581,8 +5581,8 @@
         <v>9</v>
       </c>
       <c r="I81" s="1"/>
-      <c r="J81" s="71"/>
-      <c r="K81" s="73"/>
+      <c r="J81" s="62"/>
+      <c r="K81" s="64"/>
       <c r="L81" s="41" t="s">
         <v>32</v>
       </c>
@@ -5991,7 +5991,7 @@
       </c>
     </row>
     <row r="88" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="62">
+      <c r="A88" s="68">
         <v>6</v>
       </c>
       <c r="B88" s="34" t="s">
@@ -6016,7 +6016,7 @@
         <v>12.338370174145986</v>
       </c>
       <c r="I88" s="4"/>
-      <c r="J88" s="62">
+      <c r="J88" s="68">
         <v>6</v>
       </c>
       <c r="K88" s="34" t="s">
@@ -6056,7 +6056,7 @@
       </c>
     </row>
     <row r="89" spans="1:23" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A89" s="63"/>
+      <c r="A89" s="69"/>
       <c r="B89" s="35" t="s">
         <v>16</v>
       </c>
@@ -6079,7 +6079,7 @@
         <v>11.630492226359115</v>
       </c>
       <c r="I89" s="4"/>
-      <c r="J89" s="63"/>
+      <c r="J89" s="69"/>
       <c r="K89" s="35" t="s">
         <v>16</v>
       </c>
@@ -6117,7 +6117,7 @@
       </c>
     </row>
     <row r="90" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="62">
+      <c r="A90" s="68">
         <v>7</v>
       </c>
       <c r="B90" s="32" t="s">
@@ -6142,7 +6142,7 @@
         <v>13.657987442979437</v>
       </c>
       <c r="I90" s="4"/>
-      <c r="J90" s="62">
+      <c r="J90" s="68">
         <v>7</v>
       </c>
       <c r="K90" s="32" t="s">
@@ -6182,7 +6182,7 @@
       </c>
     </row>
     <row r="91" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A91" s="64"/>
+      <c r="A91" s="70"/>
       <c r="B91" s="36" t="s">
         <v>18</v>
       </c>
@@ -6205,7 +6205,7 @@
         <v>15.194142113988185</v>
       </c>
       <c r="I91" s="4"/>
-      <c r="J91" s="64"/>
+      <c r="J91" s="70"/>
       <c r="K91" s="36" t="s">
         <v>18</v>
       </c>
@@ -6243,10 +6243,10 @@
       </c>
     </row>
     <row r="92" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="65" t="s">
+      <c r="A92" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="B92" s="66"/>
+      <c r="B92" s="72"/>
       <c r="C92" s="17">
         <v>2744.6693999999998</v>
       </c>
@@ -6266,10 +6266,10 @@
         <v>12.263709118312606</v>
       </c>
       <c r="I92" s="4"/>
-      <c r="J92" s="65" t="s">
+      <c r="J92" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="K92" s="66"/>
+      <c r="K92" s="72"/>
       <c r="L92" s="17">
         <v>2744.6693999999998</v>
       </c>
@@ -6369,16 +6369,16 @@
       </c>
     </row>
     <row r="94" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A94" s="61" t="s">
+      <c r="A94" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="B94" s="61"/>
-      <c r="C94" s="61"/>
-      <c r="D94" s="61"/>
-      <c r="E94" s="61"/>
-      <c r="F94" s="61"/>
-      <c r="G94" s="61"/>
-      <c r="H94" s="61"/>
+      <c r="B94" s="56"/>
+      <c r="C94" s="56"/>
+      <c r="D94" s="56"/>
+      <c r="E94" s="56"/>
+      <c r="F94" s="56"/>
+      <c r="G94" s="56"/>
+      <c r="H94" s="56"/>
       <c r="I94" s="1"/>
       <c r="J94" s="1"/>
       <c r="K94" s="1"/>
@@ -6396,9 +6396,9 @@
       <c r="W94" s="1"/>
     </row>
     <row r="95" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A95" s="74"/>
-      <c r="B95" s="74"/>
-      <c r="C95" s="74"/>
+      <c r="A95" s="57"/>
+      <c r="B95" s="57"/>
+      <c r="C95" s="57"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
       <c r="F95" s="3"/>
@@ -6421,16 +6421,16 @@
       <c r="W95" s="1"/>
     </row>
     <row r="96" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A96" s="67" t="s">
+      <c r="A96" s="58" t="s">
         <v>34</v>
       </c>
-      <c r="B96" s="68"/>
-      <c r="C96" s="68"/>
-      <c r="D96" s="68"/>
-      <c r="E96" s="68"/>
-      <c r="F96" s="68"/>
-      <c r="G96" s="68"/>
-      <c r="H96" s="68"/>
+      <c r="B96" s="59"/>
+      <c r="C96" s="59"/>
+      <c r="D96" s="59"/>
+      <c r="E96" s="59"/>
+      <c r="F96" s="59"/>
+      <c r="G96" s="59"/>
+      <c r="H96" s="59"/>
       <c r="I96" s="1"/>
       <c r="J96" s="1"/>
       <c r="K96" s="1"/>
@@ -6450,8 +6450,8 @@
       <c r="W96" s="1"/>
     </row>
     <row r="97" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A97" s="69"/>
-      <c r="B97" s="69"/>
+      <c r="A97" s="60"/>
+      <c r="B97" s="60"/>
       <c r="C97" s="2"/>
       <c r="D97" s="2"/>
       <c r="E97" s="2"/>
@@ -6475,35 +6475,35 @@
       <c r="W97" s="1"/>
     </row>
     <row r="98" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="70" t="s">
+      <c r="A98" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="B98" s="72" t="s">
+      <c r="B98" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="C98" s="56" t="s">
+      <c r="C98" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="D98" s="57"/>
-      <c r="E98" s="57"/>
-      <c r="F98" s="57"/>
-      <c r="G98" s="57"/>
-      <c r="H98" s="58"/>
+      <c r="D98" s="66"/>
+      <c r="E98" s="66"/>
+      <c r="F98" s="66"/>
+      <c r="G98" s="66"/>
+      <c r="H98" s="67"/>
       <c r="I98" s="1"/>
-      <c r="J98" s="70" t="s">
+      <c r="J98" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="K98" s="72" t="s">
+      <c r="K98" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="L98" s="56" t="s">
+      <c r="L98" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="M98" s="57"/>
-      <c r="N98" s="57"/>
-      <c r="O98" s="57"/>
-      <c r="P98" s="57"/>
-      <c r="Q98" s="58"/>
+      <c r="M98" s="66"/>
+      <c r="N98" s="66"/>
+      <c r="O98" s="66"/>
+      <c r="P98" s="66"/>
+      <c r="Q98" s="67"/>
       <c r="R98" s="1"/>
       <c r="S98" s="1"/>
       <c r="T98" s="1"/>
@@ -6512,35 +6512,35 @@
       <c r="W98" s="1"/>
     </row>
     <row r="99" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A99" s="71"/>
-      <c r="B99" s="73"/>
-      <c r="C99" s="59">
+      <c r="A99" s="62"/>
+      <c r="B99" s="64"/>
+      <c r="C99" s="73">
         <v>2025</v>
       </c>
-      <c r="D99" s="60"/>
-      <c r="E99" s="59">
+      <c r="D99" s="74"/>
+      <c r="E99" s="73">
         <v>2026</v>
       </c>
-      <c r="F99" s="60"/>
-      <c r="G99" s="59" t="s">
+      <c r="F99" s="74"/>
+      <c r="G99" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="H99" s="60"/>
+      <c r="H99" s="74"/>
       <c r="I99" s="1"/>
-      <c r="J99" s="71"/>
-      <c r="K99" s="73"/>
-      <c r="L99" s="59">
+      <c r="J99" s="62"/>
+      <c r="K99" s="64"/>
+      <c r="L99" s="73">
         <v>2025</v>
       </c>
-      <c r="M99" s="60"/>
-      <c r="N99" s="59">
+      <c r="M99" s="74"/>
+      <c r="N99" s="73">
         <v>2026</v>
       </c>
-      <c r="O99" s="60"/>
-      <c r="P99" s="59" t="s">
+      <c r="O99" s="74"/>
+      <c r="P99" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="Q99" s="60"/>
+      <c r="Q99" s="74"/>
       <c r="R99" s="1"/>
       <c r="S99" s="1"/>
       <c r="T99" s="1"/>
@@ -6549,8 +6549,8 @@
       <c r="W99" s="1"/>
     </row>
     <row r="100" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A100" s="71"/>
-      <c r="B100" s="73"/>
+      <c r="A100" s="62"/>
+      <c r="B100" s="64"/>
       <c r="C100" s="41" t="s">
         <v>35</v>
       </c>
@@ -6570,8 +6570,8 @@
         <v>9</v>
       </c>
       <c r="I100" s="1"/>
-      <c r="J100" s="71"/>
-      <c r="K100" s="73"/>
+      <c r="J100" s="62"/>
+      <c r="K100" s="64"/>
       <c r="L100" s="41" t="s">
         <v>35</v>
       </c>
@@ -6980,7 +6980,7 @@
       </c>
     </row>
     <row r="107" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A107" s="62">
+      <c r="A107" s="68">
         <v>6</v>
       </c>
       <c r="B107" s="34" t="s">
@@ -7005,7 +7005,7 @@
         <v>14.074469852764352</v>
       </c>
       <c r="I107" s="4"/>
-      <c r="J107" s="62">
+      <c r="J107" s="68">
         <v>6</v>
       </c>
       <c r="K107" s="34" t="s">
@@ -7045,7 +7045,7 @@
       </c>
     </row>
     <row r="108" spans="1:23" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A108" s="63"/>
+      <c r="A108" s="69"/>
       <c r="B108" s="35" t="s">
         <v>16</v>
       </c>
@@ -7068,7 +7068,7 @@
         <v>13.24554914480106</v>
       </c>
       <c r="I108" s="4"/>
-      <c r="J108" s="63"/>
+      <c r="J108" s="69"/>
       <c r="K108" s="35" t="s">
         <v>16</v>
       </c>
@@ -7106,7 +7106,7 @@
       </c>
     </row>
     <row r="109" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A109" s="62">
+      <c r="A109" s="68">
         <v>7</v>
       </c>
       <c r="B109" s="32" t="s">
@@ -7131,7 +7131,7 @@
         <v>15.755745756756442</v>
       </c>
       <c r="I109" s="4"/>
-      <c r="J109" s="62">
+      <c r="J109" s="68">
         <v>7</v>
       </c>
       <c r="K109" s="32" t="s">
@@ -7171,7 +7171,7 @@
       </c>
     </row>
     <row r="110" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A110" s="64"/>
+      <c r="A110" s="70"/>
       <c r="B110" s="36" t="s">
         <v>18</v>
       </c>
@@ -7194,7 +7194,7 @@
         <v>17.612917937465848</v>
       </c>
       <c r="I110" s="4"/>
-      <c r="J110" s="64"/>
+      <c r="J110" s="70"/>
       <c r="K110" s="36" t="s">
         <v>18</v>
       </c>
@@ -7232,10 +7232,10 @@
       </c>
     </row>
     <row r="111" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A111" s="65" t="s">
+      <c r="A111" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="B111" s="66"/>
+      <c r="B111" s="72"/>
       <c r="C111" s="17">
         <v>2650.1869999999999</v>
       </c>
@@ -7255,10 +7255,10 @@
         <v>13.963470980631238</v>
       </c>
       <c r="I111" s="4"/>
-      <c r="J111" s="65" t="s">
+      <c r="J111" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="K111" s="66"/>
+      <c r="K111" s="72"/>
       <c r="L111" s="17">
         <v>2650.1869999999999</v>
       </c>
@@ -7358,16 +7358,16 @@
       </c>
     </row>
     <row r="113" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A113" s="61" t="s">
+      <c r="A113" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="B113" s="61"/>
-      <c r="C113" s="61"/>
-      <c r="D113" s="61"/>
-      <c r="E113" s="61"/>
-      <c r="F113" s="61"/>
-      <c r="G113" s="61"/>
-      <c r="H113" s="61"/>
+      <c r="B113" s="56"/>
+      <c r="C113" s="56"/>
+      <c r="D113" s="56"/>
+      <c r="E113" s="56"/>
+      <c r="F113" s="56"/>
+      <c r="G113" s="56"/>
+      <c r="H113" s="56"/>
       <c r="I113" s="1"/>
       <c r="J113" s="1"/>
       <c r="K113" s="1"/>
@@ -7410,16 +7410,16 @@
       <c r="W114" s="1"/>
     </row>
     <row r="115" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A115" s="67" t="s">
+      <c r="A115" s="58" t="s">
         <v>37</v>
       </c>
-      <c r="B115" s="68"/>
-      <c r="C115" s="68"/>
-      <c r="D115" s="68"/>
-      <c r="E115" s="68"/>
-      <c r="F115" s="68"/>
-      <c r="G115" s="68"/>
-      <c r="H115" s="68"/>
+      <c r="B115" s="59"/>
+      <c r="C115" s="59"/>
+      <c r="D115" s="59"/>
+      <c r="E115" s="59"/>
+      <c r="F115" s="59"/>
+      <c r="G115" s="59"/>
+      <c r="H115" s="59"/>
       <c r="I115" s="1"/>
       <c r="J115" s="1"/>
       <c r="K115" s="1"/>
@@ -7439,8 +7439,8 @@
       <c r="W115" s="1"/>
     </row>
     <row r="116" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A116" s="69"/>
-      <c r="B116" s="69"/>
+      <c r="A116" s="60"/>
+      <c r="B116" s="60"/>
       <c r="C116" s="2"/>
       <c r="D116" s="2"/>
       <c r="E116" s="2"/>
@@ -7464,35 +7464,35 @@
       <c r="W116" s="1"/>
     </row>
     <row r="117" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A117" s="70" t="s">
+      <c r="A117" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="B117" s="72" t="s">
+      <c r="B117" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="C117" s="56" t="s">
+      <c r="C117" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="D117" s="57"/>
-      <c r="E117" s="57"/>
-      <c r="F117" s="57"/>
-      <c r="G117" s="57"/>
-      <c r="H117" s="58"/>
+      <c r="D117" s="66"/>
+      <c r="E117" s="66"/>
+      <c r="F117" s="66"/>
+      <c r="G117" s="66"/>
+      <c r="H117" s="67"/>
       <c r="I117" s="1"/>
-      <c r="J117" s="70" t="s">
+      <c r="J117" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="K117" s="72" t="s">
+      <c r="K117" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="L117" s="56" t="s">
+      <c r="L117" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="M117" s="57"/>
-      <c r="N117" s="57"/>
-      <c r="O117" s="57"/>
-      <c r="P117" s="57"/>
-      <c r="Q117" s="58"/>
+      <c r="M117" s="66"/>
+      <c r="N117" s="66"/>
+      <c r="O117" s="66"/>
+      <c r="P117" s="66"/>
+      <c r="Q117" s="67"/>
       <c r="R117" s="1"/>
       <c r="S117" s="1"/>
       <c r="T117" s="1"/>
@@ -7501,35 +7501,35 @@
       <c r="W117" s="1"/>
     </row>
     <row r="118" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A118" s="71"/>
-      <c r="B118" s="73"/>
-      <c r="C118" s="59">
+      <c r="A118" s="62"/>
+      <c r="B118" s="64"/>
+      <c r="C118" s="73">
         <v>2025</v>
       </c>
-      <c r="D118" s="60"/>
-      <c r="E118" s="59">
+      <c r="D118" s="74"/>
+      <c r="E118" s="73">
         <v>2026</v>
       </c>
-      <c r="F118" s="60"/>
-      <c r="G118" s="59" t="s">
+      <c r="F118" s="74"/>
+      <c r="G118" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="H118" s="60"/>
+      <c r="H118" s="74"/>
       <c r="I118" s="1"/>
-      <c r="J118" s="71"/>
-      <c r="K118" s="73"/>
-      <c r="L118" s="59">
+      <c r="J118" s="62"/>
+      <c r="K118" s="64"/>
+      <c r="L118" s="73">
         <v>2025</v>
       </c>
-      <c r="M118" s="60"/>
-      <c r="N118" s="59">
+      <c r="M118" s="74"/>
+      <c r="N118" s="73">
         <v>2026</v>
       </c>
-      <c r="O118" s="60"/>
-      <c r="P118" s="59" t="s">
+      <c r="O118" s="74"/>
+      <c r="P118" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="Q118" s="60"/>
+      <c r="Q118" s="74"/>
       <c r="R118" s="1"/>
       <c r="S118" s="1"/>
       <c r="T118" s="1"/>
@@ -7538,8 +7538,8 @@
       <c r="W118" s="1"/>
     </row>
     <row r="119" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A119" s="71"/>
-      <c r="B119" s="73"/>
+      <c r="A119" s="62"/>
+      <c r="B119" s="64"/>
       <c r="C119" s="41" t="s">
         <v>38</v>
       </c>
@@ -7559,8 +7559,8 @@
         <v>9</v>
       </c>
       <c r="I119" s="1"/>
-      <c r="J119" s="71"/>
-      <c r="K119" s="73"/>
+      <c r="J119" s="62"/>
+      <c r="K119" s="64"/>
       <c r="L119" s="41" t="s">
         <v>38</v>
       </c>
@@ -7969,7 +7969,7 @@
       </c>
     </row>
     <row r="126" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A126" s="62">
+      <c r="A126" s="68">
         <v>6</v>
       </c>
       <c r="B126" s="34" t="s">
@@ -7994,7 +7994,7 @@
         <v>16.318963869482861</v>
       </c>
       <c r="I126" s="4"/>
-      <c r="J126" s="62">
+      <c r="J126" s="68">
         <v>6</v>
       </c>
       <c r="K126" s="34" t="s">
@@ -8034,7 +8034,7 @@
       </c>
     </row>
     <row r="127" spans="1:23" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A127" s="63"/>
+      <c r="A127" s="69"/>
       <c r="B127" s="35" t="s">
         <v>16</v>
       </c>
@@ -8057,7 +8057,7 @@
         <v>15.225967824370448</v>
       </c>
       <c r="I127" s="4"/>
-      <c r="J127" s="63"/>
+      <c r="J127" s="69"/>
       <c r="K127" s="35" t="s">
         <v>16</v>
       </c>
@@ -8095,7 +8095,7 @@
       </c>
     </row>
     <row r="128" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A128" s="62">
+      <c r="A128" s="68">
         <v>7</v>
       </c>
       <c r="B128" s="32" t="s">
@@ -8120,7 +8120,7 @@
         <v>18.499610773213028</v>
       </c>
       <c r="I128" s="4"/>
-      <c r="J128" s="62">
+      <c r="J128" s="68">
         <v>7</v>
       </c>
       <c r="K128" s="32" t="s">
@@ -8160,7 +8160,7 @@
       </c>
     </row>
     <row r="129" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A129" s="64"/>
+      <c r="A129" s="70"/>
       <c r="B129" s="36" t="s">
         <v>18</v>
       </c>
@@ -8183,7 +8183,7 @@
         <v>20.724636111658011</v>
       </c>
       <c r="I129" s="4"/>
-      <c r="J129" s="64"/>
+      <c r="J129" s="70"/>
       <c r="K129" s="36" t="s">
         <v>18</v>
       </c>
@@ -8221,10 +8221,10 @@
       </c>
     </row>
     <row r="130" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A130" s="65" t="s">
+      <c r="A130" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="B130" s="66"/>
+      <c r="B130" s="72"/>
       <c r="C130" s="17">
         <v>2798.9191000000001</v>
       </c>
@@ -8244,10 +8244,10 @@
         <v>16.120931466415541</v>
       </c>
       <c r="I130" s="4"/>
-      <c r="J130" s="65" t="s">
+      <c r="J130" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="K130" s="66"/>
+      <c r="K130" s="72"/>
       <c r="L130" s="17">
         <v>2798.9191000000001</v>
       </c>
@@ -8347,16 +8347,16 @@
       </c>
     </row>
     <row r="132" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A132" s="61" t="s">
+      <c r="A132" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="B132" s="61"/>
-      <c r="C132" s="61"/>
-      <c r="D132" s="61"/>
-      <c r="E132" s="61"/>
-      <c r="F132" s="61"/>
-      <c r="G132" s="61"/>
-      <c r="H132" s="61"/>
+      <c r="B132" s="56"/>
+      <c r="C132" s="56"/>
+      <c r="D132" s="56"/>
+      <c r="E132" s="56"/>
+      <c r="F132" s="56"/>
+      <c r="G132" s="56"/>
+      <c r="H132" s="56"/>
       <c r="I132" s="1"/>
       <c r="J132" s="1"/>
       <c r="K132" s="1"/>
@@ -8374,16 +8374,16 @@
       <c r="W132" s="1"/>
     </row>
     <row r="134" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A134" s="67" t="s">
+      <c r="A134" s="58" t="s">
         <v>40</v>
       </c>
-      <c r="B134" s="68"/>
-      <c r="C134" s="68"/>
-      <c r="D134" s="68"/>
-      <c r="E134" s="68"/>
-      <c r="F134" s="68"/>
-      <c r="G134" s="68"/>
-      <c r="H134" s="68"/>
+      <c r="B134" s="59"/>
+      <c r="C134" s="59"/>
+      <c r="D134" s="59"/>
+      <c r="E134" s="59"/>
+      <c r="F134" s="59"/>
+      <c r="G134" s="59"/>
+      <c r="H134" s="59"/>
       <c r="I134" s="1"/>
       <c r="J134" s="1"/>
       <c r="K134" s="1"/>
@@ -8403,8 +8403,8 @@
       <c r="W134" s="1"/>
     </row>
     <row r="135" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A135" s="69"/>
-      <c r="B135" s="69"/>
+      <c r="A135" s="60"/>
+      <c r="B135" s="60"/>
       <c r="C135" s="2"/>
       <c r="D135" s="2"/>
       <c r="E135" s="2"/>
@@ -8428,35 +8428,35 @@
       <c r="W135" s="1"/>
     </row>
     <row r="136" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A136" s="70" t="s">
+      <c r="A136" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="B136" s="72" t="s">
+      <c r="B136" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="C136" s="56" t="s">
+      <c r="C136" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="D136" s="57"/>
-      <c r="E136" s="57"/>
-      <c r="F136" s="57"/>
-      <c r="G136" s="57"/>
-      <c r="H136" s="58"/>
+      <c r="D136" s="66"/>
+      <c r="E136" s="66"/>
+      <c r="F136" s="66"/>
+      <c r="G136" s="66"/>
+      <c r="H136" s="67"/>
       <c r="I136" s="1"/>
-      <c r="J136" s="70" t="s">
+      <c r="J136" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="K136" s="72" t="s">
+      <c r="K136" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="L136" s="56" t="s">
+      <c r="L136" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="M136" s="57"/>
-      <c r="N136" s="57"/>
-      <c r="O136" s="57"/>
-      <c r="P136" s="57"/>
-      <c r="Q136" s="58"/>
+      <c r="M136" s="66"/>
+      <c r="N136" s="66"/>
+      <c r="O136" s="66"/>
+      <c r="P136" s="66"/>
+      <c r="Q136" s="67"/>
       <c r="R136" s="1"/>
       <c r="S136" s="1"/>
       <c r="T136" s="1"/>
@@ -8465,35 +8465,35 @@
       <c r="W136" s="1"/>
     </row>
     <row r="137" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A137" s="71"/>
-      <c r="B137" s="73"/>
-      <c r="C137" s="59">
+      <c r="A137" s="62"/>
+      <c r="B137" s="64"/>
+      <c r="C137" s="73">
         <v>2025</v>
       </c>
-      <c r="D137" s="60"/>
-      <c r="E137" s="59">
+      <c r="D137" s="74"/>
+      <c r="E137" s="73">
         <v>2026</v>
       </c>
-      <c r="F137" s="60"/>
-      <c r="G137" s="59" t="s">
+      <c r="F137" s="74"/>
+      <c r="G137" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="H137" s="60"/>
+      <c r="H137" s="74"/>
       <c r="I137" s="1"/>
-      <c r="J137" s="71"/>
-      <c r="K137" s="73"/>
-      <c r="L137" s="59">
+      <c r="J137" s="62"/>
+      <c r="K137" s="64"/>
+      <c r="L137" s="73">
         <v>2025</v>
       </c>
-      <c r="M137" s="60"/>
-      <c r="N137" s="59">
+      <c r="M137" s="74"/>
+      <c r="N137" s="73">
         <v>2026</v>
       </c>
-      <c r="O137" s="60"/>
-      <c r="P137" s="59" t="s">
+      <c r="O137" s="74"/>
+      <c r="P137" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="Q137" s="60"/>
+      <c r="Q137" s="74"/>
       <c r="R137" s="1"/>
       <c r="S137" s="1"/>
       <c r="T137" s="1"/>
@@ -8502,8 +8502,8 @@
       <c r="W137" s="1"/>
     </row>
     <row r="138" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A138" s="71"/>
-      <c r="B138" s="73"/>
+      <c r="A138" s="62"/>
+      <c r="B138" s="64"/>
       <c r="C138" s="41" t="s">
         <v>41</v>
       </c>
@@ -8523,8 +8523,8 @@
         <v>9</v>
       </c>
       <c r="I138" s="1"/>
-      <c r="J138" s="71"/>
-      <c r="K138" s="73"/>
+      <c r="J138" s="62"/>
+      <c r="K138" s="64"/>
       <c r="L138" s="41" t="s">
         <v>41</v>
       </c>
@@ -8933,7 +8933,7 @@
       </c>
     </row>
     <row r="145" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A145" s="62">
+      <c r="A145" s="68">
         <v>6</v>
       </c>
       <c r="B145" s="34" t="s">
@@ -8958,7 +8958,7 @@
         <v>19.677766681341584</v>
       </c>
       <c r="I145" s="4"/>
-      <c r="J145" s="62">
+      <c r="J145" s="68">
         <v>6</v>
       </c>
       <c r="K145" s="34" t="s">
@@ -8998,7 +8998,7 @@
       </c>
     </row>
     <row r="146" spans="1:23" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A146" s="63"/>
+      <c r="A146" s="69"/>
       <c r="B146" s="35" t="s">
         <v>16</v>
       </c>
@@ -9021,7 +9021,7 @@
         <v>18.419792372051987</v>
       </c>
       <c r="I146" s="4"/>
-      <c r="J146" s="63"/>
+      <c r="J146" s="69"/>
       <c r="K146" s="35" t="s">
         <v>16</v>
       </c>
@@ -9059,7 +9059,7 @@
       </c>
     </row>
     <row r="147" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A147" s="62">
+      <c r="A147" s="68">
         <v>7</v>
       </c>
       <c r="B147" s="32" t="s">
@@ -9084,7 +9084,7 @@
         <v>21.927704528535109</v>
       </c>
       <c r="I147" s="4"/>
-      <c r="J147" s="62">
+      <c r="J147" s="68">
         <v>7</v>
       </c>
       <c r="K147" s="32" t="s">
@@ -9124,7 +9124,7 @@
       </c>
     </row>
     <row r="148" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A148" s="64"/>
+      <c r="A148" s="70"/>
       <c r="B148" s="36" t="s">
         <v>18</v>
       </c>
@@ -9147,7 +9147,7 @@
         <v>24.587108361222271</v>
       </c>
       <c r="I148" s="4"/>
-      <c r="J148" s="64"/>
+      <c r="J148" s="70"/>
       <c r="K148" s="36" t="s">
         <v>18</v>
       </c>
@@ -9185,10 +9185,10 @@
       </c>
     </row>
     <row r="149" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A149" s="65" t="s">
+      <c r="A149" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="B149" s="66"/>
+      <c r="B149" s="72"/>
       <c r="C149" s="17">
         <v>2916.9663999999998</v>
       </c>
@@ -9208,10 +9208,10 @@
         <v>19.264483553919863</v>
       </c>
       <c r="I149" s="4"/>
-      <c r="J149" s="65" t="s">
+      <c r="J149" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="K149" s="66"/>
+      <c r="K149" s="72"/>
       <c r="L149" s="17">
         <v>2916.9663999999993</v>
       </c>
@@ -9311,16 +9311,16 @@
       </c>
     </row>
     <row r="151" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A151" s="61" t="s">
+      <c r="A151" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="B151" s="61"/>
-      <c r="C151" s="61"/>
-      <c r="D151" s="61"/>
-      <c r="E151" s="61"/>
-      <c r="F151" s="61"/>
-      <c r="G151" s="61"/>
-      <c r="H151" s="61"/>
+      <c r="B151" s="56"/>
+      <c r="C151" s="56"/>
+      <c r="D151" s="56"/>
+      <c r="E151" s="56"/>
+      <c r="F151" s="56"/>
+      <c r="G151" s="56"/>
+      <c r="H151" s="56"/>
       <c r="I151" s="1"/>
       <c r="J151" s="1"/>
       <c r="K151" s="1"/>
@@ -9338,16 +9338,16 @@
       <c r="W151" s="1"/>
     </row>
     <row r="153" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A153" s="67" t="s">
+      <c r="A153" s="58" t="s">
         <v>43</v>
       </c>
-      <c r="B153" s="68"/>
-      <c r="C153" s="68"/>
-      <c r="D153" s="68"/>
-      <c r="E153" s="68"/>
-      <c r="F153" s="68"/>
-      <c r="G153" s="68"/>
-      <c r="H153" s="68"/>
+      <c r="B153" s="59"/>
+      <c r="C153" s="59"/>
+      <c r="D153" s="59"/>
+      <c r="E153" s="59"/>
+      <c r="F153" s="59"/>
+      <c r="G153" s="59"/>
+      <c r="H153" s="59"/>
       <c r="I153" s="1"/>
       <c r="J153" s="1"/>
       <c r="K153" s="1"/>
@@ -9367,8 +9367,8 @@
       <c r="W153" s="1"/>
     </row>
     <row r="154" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A154" s="69"/>
-      <c r="B154" s="69"/>
+      <c r="A154" s="60"/>
+      <c r="B154" s="60"/>
       <c r="C154" s="2"/>
       <c r="D154" s="2"/>
       <c r="E154" s="2"/>
@@ -9392,35 +9392,35 @@
       <c r="W154" s="1"/>
     </row>
     <row r="155" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A155" s="70" t="s">
+      <c r="A155" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="B155" s="72" t="s">
+      <c r="B155" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="C155" s="56" t="s">
+      <c r="C155" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="D155" s="57"/>
-      <c r="E155" s="57"/>
-      <c r="F155" s="57"/>
-      <c r="G155" s="57"/>
-      <c r="H155" s="58"/>
+      <c r="D155" s="66"/>
+      <c r="E155" s="66"/>
+      <c r="F155" s="66"/>
+      <c r="G155" s="66"/>
+      <c r="H155" s="67"/>
       <c r="I155" s="1"/>
-      <c r="J155" s="70" t="s">
+      <c r="J155" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="K155" s="72" t="s">
+      <c r="K155" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="L155" s="56" t="s">
+      <c r="L155" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="M155" s="57"/>
-      <c r="N155" s="57"/>
-      <c r="O155" s="57"/>
-      <c r="P155" s="57"/>
-      <c r="Q155" s="58"/>
+      <c r="M155" s="66"/>
+      <c r="N155" s="66"/>
+      <c r="O155" s="66"/>
+      <c r="P155" s="66"/>
+      <c r="Q155" s="67"/>
       <c r="R155" s="1"/>
       <c r="S155" s="1"/>
       <c r="T155" s="1"/>
@@ -9429,35 +9429,35 @@
       <c r="W155" s="1"/>
     </row>
     <row r="156" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A156" s="71"/>
-      <c r="B156" s="73"/>
-      <c r="C156" s="59">
+      <c r="A156" s="62"/>
+      <c r="B156" s="64"/>
+      <c r="C156" s="73">
         <v>2025</v>
       </c>
-      <c r="D156" s="60"/>
-      <c r="E156" s="59">
+      <c r="D156" s="74"/>
+      <c r="E156" s="73">
         <v>2026</v>
       </c>
-      <c r="F156" s="60"/>
-      <c r="G156" s="59" t="s">
+      <c r="F156" s="74"/>
+      <c r="G156" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="H156" s="60"/>
+      <c r="H156" s="74"/>
       <c r="I156" s="1"/>
-      <c r="J156" s="71"/>
-      <c r="K156" s="73"/>
-      <c r="L156" s="59">
+      <c r="J156" s="62"/>
+      <c r="K156" s="64"/>
+      <c r="L156" s="73">
         <v>2025</v>
       </c>
-      <c r="M156" s="60"/>
-      <c r="N156" s="59">
+      <c r="M156" s="74"/>
+      <c r="N156" s="73">
         <v>2026</v>
       </c>
-      <c r="O156" s="60"/>
-      <c r="P156" s="59" t="s">
+      <c r="O156" s="74"/>
+      <c r="P156" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="Q156" s="60"/>
+      <c r="Q156" s="74"/>
       <c r="R156" s="1"/>
       <c r="S156" s="1"/>
       <c r="T156" s="1"/>
@@ -9466,8 +9466,8 @@
       <c r="W156" s="1"/>
     </row>
     <row r="157" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A157" s="71"/>
-      <c r="B157" s="73"/>
+      <c r="A157" s="62"/>
+      <c r="B157" s="64"/>
       <c r="C157" s="41" t="s">
         <v>44</v>
       </c>
@@ -9487,8 +9487,8 @@
         <v>9</v>
       </c>
       <c r="I157" s="1"/>
-      <c r="J157" s="71"/>
-      <c r="K157" s="73"/>
+      <c r="J157" s="62"/>
+      <c r="K157" s="64"/>
       <c r="L157" s="41" t="s">
         <v>44</v>
       </c>
@@ -9897,7 +9897,7 @@
       </c>
     </row>
     <row r="164" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A164" s="62">
+      <c r="A164" s="68">
         <v>6</v>
       </c>
       <c r="B164" s="34" t="s">
@@ -9922,7 +9922,7 @@
         <v>24.985700708174789</v>
       </c>
       <c r="I164" s="4"/>
-      <c r="J164" s="62">
+      <c r="J164" s="68">
         <v>6</v>
       </c>
       <c r="K164" s="34" t="s">
@@ -9962,7 +9962,7 @@
       </c>
     </row>
     <row r="165" spans="1:23" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A165" s="63"/>
+      <c r="A165" s="69"/>
       <c r="B165" s="35" t="s">
         <v>16</v>
       </c>
@@ -9985,7 +9985,7 @@
         <v>23.348552308059155</v>
       </c>
       <c r="I165" s="4"/>
-      <c r="J165" s="63"/>
+      <c r="J165" s="69"/>
       <c r="K165" s="35" t="s">
         <v>16</v>
       </c>
@@ -10023,7 +10023,7 @@
       </c>
     </row>
     <row r="166" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A166" s="62">
+      <c r="A166" s="68">
         <v>7</v>
       </c>
       <c r="B166" s="32" t="s">
@@ -10048,7 +10048,7 @@
         <v>27.540934419202745</v>
       </c>
       <c r="I166" s="4"/>
-      <c r="J166" s="62">
+      <c r="J166" s="68">
         <v>7</v>
       </c>
       <c r="K166" s="32" t="s">
@@ -10088,7 +10088,7 @@
       </c>
     </row>
     <row r="167" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A167" s="64"/>
+      <c r="A167" s="70"/>
       <c r="B167" s="36" t="s">
         <v>18</v>
       </c>
@@ -10111,7 +10111,7 @@
         <v>31.063872604239211</v>
       </c>
       <c r="I167" s="4"/>
-      <c r="J167" s="64"/>
+      <c r="J167" s="70"/>
       <c r="K167" s="36" t="s">
         <v>18</v>
       </c>
@@ -10149,10 +10149,10 @@
       </c>
     </row>
     <row r="168" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A168" s="65" t="s">
+      <c r="A168" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="B168" s="66"/>
+      <c r="B168" s="72"/>
       <c r="C168" s="17">
         <v>2874.1851999999999</v>
       </c>
@@ -10172,10 +10172,10 @@
         <v>24.177993882412505</v>
       </c>
       <c r="I168" s="4"/>
-      <c r="J168" s="65" t="s">
+      <c r="J168" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="K168" s="66"/>
+      <c r="K168" s="72"/>
       <c r="L168" s="17">
         <v>2874.1851999999999</v>
       </c>
@@ -10275,16 +10275,16 @@
       </c>
     </row>
     <row r="170" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A170" s="61" t="s">
+      <c r="A170" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="B170" s="61"/>
-      <c r="C170" s="61"/>
-      <c r="D170" s="61"/>
-      <c r="E170" s="61"/>
-      <c r="F170" s="61"/>
-      <c r="G170" s="61"/>
-      <c r="H170" s="61"/>
+      <c r="B170" s="56"/>
+      <c r="C170" s="56"/>
+      <c r="D170" s="56"/>
+      <c r="E170" s="56"/>
+      <c r="F170" s="56"/>
+      <c r="G170" s="56"/>
+      <c r="H170" s="56"/>
       <c r="I170" s="1"/>
       <c r="J170" s="1"/>
       <c r="K170" s="1"/>
@@ -10302,16 +10302,16 @@
       <c r="W170" s="1"/>
     </row>
     <row r="172" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A172" s="67" t="s">
+      <c r="A172" s="58" t="s">
         <v>46</v>
       </c>
-      <c r="B172" s="68"/>
-      <c r="C172" s="68"/>
-      <c r="D172" s="68"/>
-      <c r="E172" s="68"/>
-      <c r="F172" s="68"/>
-      <c r="G172" s="68"/>
-      <c r="H172" s="68"/>
+      <c r="B172" s="59"/>
+      <c r="C172" s="59"/>
+      <c r="D172" s="59"/>
+      <c r="E172" s="59"/>
+      <c r="F172" s="59"/>
+      <c r="G172" s="59"/>
+      <c r="H172" s="59"/>
       <c r="I172" s="1"/>
       <c r="J172" s="1"/>
       <c r="K172" s="1"/>
@@ -10331,8 +10331,8 @@
       <c r="W172" s="1"/>
     </row>
     <row r="173" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A173" s="69"/>
-      <c r="B173" s="69"/>
+      <c r="A173" s="60"/>
+      <c r="B173" s="60"/>
       <c r="C173" s="2"/>
       <c r="D173" s="2"/>
       <c r="E173" s="2"/>
@@ -10356,35 +10356,35 @@
       <c r="W173" s="1"/>
     </row>
     <row r="174" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A174" s="70" t="s">
+      <c r="A174" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="B174" s="72" t="s">
+      <c r="B174" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="C174" s="56" t="s">
+      <c r="C174" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="D174" s="57"/>
-      <c r="E174" s="57"/>
-      <c r="F174" s="57"/>
-      <c r="G174" s="57"/>
-      <c r="H174" s="58"/>
+      <c r="D174" s="66"/>
+      <c r="E174" s="66"/>
+      <c r="F174" s="66"/>
+      <c r="G174" s="66"/>
+      <c r="H174" s="67"/>
       <c r="I174" s="1"/>
-      <c r="J174" s="70" t="s">
+      <c r="J174" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="K174" s="72" t="s">
+      <c r="K174" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="L174" s="56" t="s">
+      <c r="L174" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="M174" s="57"/>
-      <c r="N174" s="57"/>
-      <c r="O174" s="57"/>
-      <c r="P174" s="57"/>
-      <c r="Q174" s="58"/>
+      <c r="M174" s="66"/>
+      <c r="N174" s="66"/>
+      <c r="O174" s="66"/>
+      <c r="P174" s="66"/>
+      <c r="Q174" s="67"/>
       <c r="R174" s="1"/>
       <c r="S174" s="1"/>
       <c r="T174" s="1"/>
@@ -10393,35 +10393,35 @@
       <c r="W174" s="1"/>
     </row>
     <row r="175" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A175" s="71"/>
-      <c r="B175" s="73"/>
-      <c r="C175" s="59">
+      <c r="A175" s="62"/>
+      <c r="B175" s="64"/>
+      <c r="C175" s="73">
         <v>2025</v>
       </c>
-      <c r="D175" s="60"/>
-      <c r="E175" s="59">
+      <c r="D175" s="74"/>
+      <c r="E175" s="73">
         <v>2026</v>
       </c>
-      <c r="F175" s="60"/>
-      <c r="G175" s="59" t="s">
+      <c r="F175" s="74"/>
+      <c r="G175" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="H175" s="60"/>
+      <c r="H175" s="74"/>
       <c r="I175" s="1"/>
-      <c r="J175" s="71"/>
-      <c r="K175" s="73"/>
-      <c r="L175" s="59">
+      <c r="J175" s="62"/>
+      <c r="K175" s="64"/>
+      <c r="L175" s="73">
         <v>2025</v>
       </c>
-      <c r="M175" s="60"/>
-      <c r="N175" s="59">
+      <c r="M175" s="74"/>
+      <c r="N175" s="73">
         <v>2026</v>
       </c>
-      <c r="O175" s="60"/>
-      <c r="P175" s="59" t="s">
+      <c r="O175" s="74"/>
+      <c r="P175" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="Q175" s="60"/>
+      <c r="Q175" s="74"/>
       <c r="R175" s="1"/>
       <c r="S175" s="1"/>
       <c r="T175" s="1"/>
@@ -10430,8 +10430,8 @@
       <c r="W175" s="1"/>
     </row>
     <row r="176" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A176" s="71"/>
-      <c r="B176" s="73"/>
+      <c r="A176" s="62"/>
+      <c r="B176" s="64"/>
       <c r="C176" s="41" t="s">
         <v>47</v>
       </c>
@@ -10451,8 +10451,8 @@
         <v>9</v>
       </c>
       <c r="I176" s="1"/>
-      <c r="J176" s="71"/>
-      <c r="K176" s="73"/>
+      <c r="J176" s="62"/>
+      <c r="K176" s="64"/>
       <c r="L176" s="41" t="s">
         <v>47</v>
       </c>
@@ -10861,7 +10861,7 @@
       </c>
     </row>
     <row r="183" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A183" s="62">
+      <c r="A183" s="68">
         <v>6</v>
       </c>
       <c r="B183" s="34" t="s">
@@ -10886,7 +10886,7 @@
         <v>33.510433646988169</v>
       </c>
       <c r="I183" s="4"/>
-      <c r="J183" s="62">
+      <c r="J183" s="68">
         <v>6</v>
       </c>
       <c r="K183" s="34" t="s">
@@ -10926,7 +10926,7 @@
       </c>
     </row>
     <row r="184" spans="1:23" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A184" s="63"/>
+      <c r="A184" s="69"/>
       <c r="B184" s="35" t="s">
         <v>16</v>
       </c>
@@ -10949,7 +10949,7 @@
         <v>31.320888282950111</v>
       </c>
       <c r="I184" s="4"/>
-      <c r="J184" s="63"/>
+      <c r="J184" s="69"/>
       <c r="K184" s="35" t="s">
         <v>16</v>
       </c>
@@ -10987,7 +10987,7 @@
       </c>
     </row>
     <row r="185" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A185" s="62">
+      <c r="A185" s="68">
         <v>7</v>
       </c>
       <c r="B185" s="32" t="s">
@@ -11012,7 +11012,7 @@
         <v>36.345396300823928</v>
       </c>
       <c r="I185" s="4"/>
-      <c r="J185" s="62">
+      <c r="J185" s="68">
         <v>7</v>
       </c>
       <c r="K185" s="32" t="s">
@@ -11052,7 +11052,7 @@
       </c>
     </row>
     <row r="186" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A186" s="64"/>
+      <c r="A186" s="70"/>
       <c r="B186" s="36" t="s">
         <v>18</v>
       </c>
@@ -11075,7 +11075,7 @@
         <v>40.312403915221665</v>
       </c>
       <c r="I186" s="4"/>
-      <c r="J186" s="64"/>
+      <c r="J186" s="70"/>
       <c r="K186" s="36" t="s">
         <v>18</v>
       </c>
@@ -11113,10 +11113,10 @@
       </c>
     </row>
     <row r="187" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A187" s="65" t="s">
+      <c r="A187" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="B187" s="66"/>
+      <c r="B187" s="72"/>
       <c r="C187" s="17">
         <v>3162.0996000000005</v>
       </c>
@@ -11136,10 +11136,10 @@
         <v>32.293932601675237</v>
       </c>
       <c r="I187" s="4"/>
-      <c r="J187" s="65" t="s">
+      <c r="J187" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="K187" s="66"/>
+      <c r="K187" s="72"/>
       <c r="L187" s="17">
         <v>3162.0996000000005</v>
       </c>
@@ -11239,16 +11239,16 @@
       </c>
     </row>
     <row r="189" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A189" s="61" t="s">
+      <c r="A189" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="B189" s="61"/>
-      <c r="C189" s="61"/>
-      <c r="D189" s="61"/>
-      <c r="E189" s="61"/>
-      <c r="F189" s="61"/>
-      <c r="G189" s="61"/>
-      <c r="H189" s="61"/>
+      <c r="B189" s="56"/>
+      <c r="C189" s="56"/>
+      <c r="D189" s="56"/>
+      <c r="E189" s="56"/>
+      <c r="F189" s="56"/>
+      <c r="G189" s="56"/>
+      <c r="H189" s="56"/>
       <c r="I189" s="1"/>
       <c r="J189" s="1"/>
       <c r="K189" s="1"/>
@@ -11266,16 +11266,16 @@
       <c r="W189" s="1"/>
     </row>
     <row r="191" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A191" s="67" t="s">
+      <c r="A191" s="58" t="s">
         <v>49</v>
       </c>
-      <c r="B191" s="68"/>
-      <c r="C191" s="68"/>
-      <c r="D191" s="68"/>
-      <c r="E191" s="68"/>
-      <c r="F191" s="68"/>
-      <c r="G191" s="68"/>
-      <c r="H191" s="68"/>
+      <c r="B191" s="59"/>
+      <c r="C191" s="59"/>
+      <c r="D191" s="59"/>
+      <c r="E191" s="59"/>
+      <c r="F191" s="59"/>
+      <c r="G191" s="59"/>
+      <c r="H191" s="59"/>
       <c r="I191" s="1"/>
       <c r="J191" s="1"/>
       <c r="K191" s="1"/>
@@ -11295,8 +11295,8 @@
       <c r="W191" s="1"/>
     </row>
     <row r="192" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A192" s="69"/>
-      <c r="B192" s="69"/>
+      <c r="A192" s="60"/>
+      <c r="B192" s="60"/>
       <c r="C192" s="2"/>
       <c r="D192" s="2"/>
       <c r="E192" s="2"/>
@@ -11320,35 +11320,35 @@
       <c r="W192" s="1"/>
     </row>
     <row r="193" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A193" s="70" t="s">
+      <c r="A193" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="B193" s="72" t="s">
+      <c r="B193" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="C193" s="56" t="s">
+      <c r="C193" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="D193" s="57"/>
-      <c r="E193" s="57"/>
-      <c r="F193" s="57"/>
-      <c r="G193" s="57"/>
-      <c r="H193" s="58"/>
+      <c r="D193" s="66"/>
+      <c r="E193" s="66"/>
+      <c r="F193" s="66"/>
+      <c r="G193" s="66"/>
+      <c r="H193" s="67"/>
       <c r="I193" s="1"/>
-      <c r="J193" s="70" t="s">
+      <c r="J193" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="K193" s="72" t="s">
+      <c r="K193" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="L193" s="56" t="s">
+      <c r="L193" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="M193" s="57"/>
-      <c r="N193" s="57"/>
-      <c r="O193" s="57"/>
-      <c r="P193" s="57"/>
-      <c r="Q193" s="58"/>
+      <c r="M193" s="66"/>
+      <c r="N193" s="66"/>
+      <c r="O193" s="66"/>
+      <c r="P193" s="66"/>
+      <c r="Q193" s="67"/>
       <c r="R193" s="1"/>
       <c r="S193" s="1"/>
       <c r="T193" s="1"/>
@@ -11357,35 +11357,35 @@
       <c r="W193" s="1"/>
     </row>
     <row r="194" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A194" s="71"/>
-      <c r="B194" s="73"/>
-      <c r="C194" s="59">
+      <c r="A194" s="62"/>
+      <c r="B194" s="64"/>
+      <c r="C194" s="73">
         <v>2025</v>
       </c>
-      <c r="D194" s="60"/>
-      <c r="E194" s="59">
+      <c r="D194" s="74"/>
+      <c r="E194" s="73">
         <v>2026</v>
       </c>
-      <c r="F194" s="60"/>
-      <c r="G194" s="59" t="s">
+      <c r="F194" s="74"/>
+      <c r="G194" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="H194" s="60"/>
+      <c r="H194" s="74"/>
       <c r="I194" s="1"/>
-      <c r="J194" s="71"/>
-      <c r="K194" s="73"/>
-      <c r="L194" s="59">
+      <c r="J194" s="62"/>
+      <c r="K194" s="64"/>
+      <c r="L194" s="73">
         <v>2025</v>
       </c>
-      <c r="M194" s="60"/>
-      <c r="N194" s="59">
+      <c r="M194" s="74"/>
+      <c r="N194" s="73">
         <v>2026</v>
       </c>
-      <c r="O194" s="60"/>
-      <c r="P194" s="59" t="s">
+      <c r="O194" s="74"/>
+      <c r="P194" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="Q194" s="60"/>
+      <c r="Q194" s="74"/>
       <c r="R194" s="1"/>
       <c r="S194" s="1"/>
       <c r="T194" s="1"/>
@@ -11394,8 +11394,8 @@
       <c r="W194" s="1"/>
     </row>
     <row r="195" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A195" s="71"/>
-      <c r="B195" s="73"/>
+      <c r="A195" s="62"/>
+      <c r="B195" s="64"/>
       <c r="C195" s="41" t="s">
         <v>50</v>
       </c>
@@ -11415,8 +11415,8 @@
         <v>9</v>
       </c>
       <c r="I195" s="1"/>
-      <c r="J195" s="71"/>
-      <c r="K195" s="73"/>
+      <c r="J195" s="62"/>
+      <c r="K195" s="64"/>
       <c r="L195" s="41" t="s">
         <v>50</v>
       </c>
@@ -11825,7 +11825,7 @@
       </c>
     </row>
     <row r="202" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A202" s="62">
+      <c r="A202" s="68">
         <v>6</v>
       </c>
       <c r="B202" s="34" t="s">
@@ -11850,7 +11850,7 @@
         <v>53.467496502995068</v>
       </c>
       <c r="I202" s="4"/>
-      <c r="J202" s="62">
+      <c r="J202" s="68">
         <v>6</v>
       </c>
       <c r="K202" s="34" t="s">
@@ -11890,7 +11890,7 @@
       </c>
     </row>
     <row r="203" spans="1:23" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A203" s="63"/>
+      <c r="A203" s="69"/>
       <c r="B203" s="35" t="s">
         <v>16</v>
       </c>
@@ -11913,7 +11913,7 @@
         <v>49.07267906380855</v>
       </c>
       <c r="I203" s="4"/>
-      <c r="J203" s="63"/>
+      <c r="J203" s="69"/>
       <c r="K203" s="35" t="s">
         <v>16</v>
       </c>
@@ -11951,7 +11951,7 @@
       </c>
     </row>
     <row r="204" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A204" s="62">
+      <c r="A204" s="68">
         <v>7</v>
       </c>
       <c r="B204" s="32" t="s">
@@ -11976,7 +11976,7 @@
         <v>59.515520179170714</v>
       </c>
       <c r="I204" s="4"/>
-      <c r="J204" s="62">
+      <c r="J204" s="68">
         <v>7</v>
       </c>
       <c r="K204" s="32" t="s">
@@ -12016,7 +12016,7 @@
       </c>
     </row>
     <row r="205" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A205" s="64"/>
+      <c r="A205" s="70"/>
       <c r="B205" s="36" t="s">
         <v>18</v>
       </c>
@@ -12039,7 +12039,7 @@
         <v>69.072705763298103</v>
       </c>
       <c r="I205" s="4"/>
-      <c r="J205" s="64"/>
+      <c r="J205" s="70"/>
       <c r="K205" s="36" t="s">
         <v>18</v>
       </c>
@@ -12077,10 +12077,10 @@
       </c>
     </row>
     <row r="206" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A206" s="65" t="s">
+      <c r="A206" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="B206" s="66"/>
+      <c r="B206" s="72"/>
       <c r="C206" s="17">
         <v>2624.9187999999995</v>
       </c>
@@ -12100,10 +12100,10 @@
         <v>51.203316843554489</v>
       </c>
       <c r="I206" s="4"/>
-      <c r="J206" s="65" t="s">
+      <c r="J206" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="K206" s="66"/>
+      <c r="K206" s="72"/>
       <c r="L206" s="17">
         <v>2624.9187999999995</v>
       </c>
@@ -12203,16 +12203,16 @@
       </c>
     </row>
     <row r="208" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A208" s="61" t="s">
+      <c r="A208" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="B208" s="61"/>
-      <c r="C208" s="61"/>
-      <c r="D208" s="61"/>
-      <c r="E208" s="61"/>
-      <c r="F208" s="61"/>
-      <c r="G208" s="61"/>
-      <c r="H208" s="61"/>
+      <c r="B208" s="56"/>
+      <c r="C208" s="56"/>
+      <c r="D208" s="56"/>
+      <c r="E208" s="56"/>
+      <c r="F208" s="56"/>
+      <c r="G208" s="56"/>
+      <c r="H208" s="56"/>
       <c r="I208" s="1"/>
       <c r="J208" s="1"/>
       <c r="K208" s="1"/>
@@ -12230,16 +12230,16 @@
       <c r="W208" s="1"/>
     </row>
     <row r="210" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A210" s="67" t="s">
+      <c r="A210" s="58" t="s">
         <v>52</v>
       </c>
-      <c r="B210" s="68"/>
-      <c r="C210" s="68"/>
-      <c r="D210" s="68"/>
-      <c r="E210" s="68"/>
-      <c r="F210" s="68"/>
-      <c r="G210" s="68"/>
-      <c r="H210" s="68"/>
+      <c r="B210" s="59"/>
+      <c r="C210" s="59"/>
+      <c r="D210" s="59"/>
+      <c r="E210" s="59"/>
+      <c r="F210" s="59"/>
+      <c r="G210" s="59"/>
+      <c r="H210" s="59"/>
       <c r="I210" s="1"/>
       <c r="J210" s="1"/>
       <c r="K210" s="1"/>
@@ -12259,8 +12259,8 @@
       <c r="W210" s="1"/>
     </row>
     <row r="211" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A211" s="69"/>
-      <c r="B211" s="69"/>
+      <c r="A211" s="60"/>
+      <c r="B211" s="60"/>
       <c r="C211" s="2"/>
       <c r="D211" s="2"/>
       <c r="E211" s="2"/>
@@ -12284,35 +12284,35 @@
       <c r="W211" s="1"/>
     </row>
     <row r="212" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A212" s="70" t="s">
+      <c r="A212" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="B212" s="72" t="s">
+      <c r="B212" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="C212" s="56" t="s">
+      <c r="C212" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="D212" s="57"/>
-      <c r="E212" s="57"/>
-      <c r="F212" s="57"/>
-      <c r="G212" s="57"/>
-      <c r="H212" s="58"/>
+      <c r="D212" s="66"/>
+      <c r="E212" s="66"/>
+      <c r="F212" s="66"/>
+      <c r="G212" s="66"/>
+      <c r="H212" s="67"/>
       <c r="I212" s="1"/>
-      <c r="J212" s="70" t="s">
+      <c r="J212" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="K212" s="72" t="s">
+      <c r="K212" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="L212" s="56" t="s">
+      <c r="L212" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="M212" s="57"/>
-      <c r="N212" s="57"/>
-      <c r="O212" s="57"/>
-      <c r="P212" s="57"/>
-      <c r="Q212" s="58"/>
+      <c r="M212" s="66"/>
+      <c r="N212" s="66"/>
+      <c r="O212" s="66"/>
+      <c r="P212" s="66"/>
+      <c r="Q212" s="67"/>
       <c r="R212" s="1"/>
       <c r="S212" s="1"/>
       <c r="T212" s="1"/>
@@ -12321,35 +12321,35 @@
       <c r="W212" s="1"/>
     </row>
     <row r="213" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A213" s="71"/>
-      <c r="B213" s="73"/>
-      <c r="C213" s="59">
+      <c r="A213" s="62"/>
+      <c r="B213" s="64"/>
+      <c r="C213" s="73">
         <v>2025</v>
       </c>
-      <c r="D213" s="60"/>
-      <c r="E213" s="59">
+      <c r="D213" s="74"/>
+      <c r="E213" s="73">
         <v>2026</v>
       </c>
-      <c r="F213" s="60"/>
-      <c r="G213" s="59" t="s">
+      <c r="F213" s="74"/>
+      <c r="G213" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="H213" s="60"/>
+      <c r="H213" s="74"/>
       <c r="I213" s="1"/>
-      <c r="J213" s="71"/>
-      <c r="K213" s="73"/>
-      <c r="L213" s="59">
+      <c r="J213" s="62"/>
+      <c r="K213" s="64"/>
+      <c r="L213" s="73">
         <v>2025</v>
       </c>
-      <c r="M213" s="60"/>
-      <c r="N213" s="59">
+      <c r="M213" s="74"/>
+      <c r="N213" s="73">
         <v>2026</v>
       </c>
-      <c r="O213" s="60"/>
-      <c r="P213" s="59" t="s">
+      <c r="O213" s="74"/>
+      <c r="P213" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="Q213" s="60"/>
+      <c r="Q213" s="74"/>
       <c r="R213" s="1"/>
       <c r="S213" s="1"/>
       <c r="T213" s="1"/>
@@ -12358,8 +12358,8 @@
       <c r="W213" s="1"/>
     </row>
     <row r="214" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A214" s="71"/>
-      <c r="B214" s="73"/>
+      <c r="A214" s="62"/>
+      <c r="B214" s="64"/>
       <c r="C214" s="41" t="s">
         <v>53</v>
       </c>
@@ -12379,8 +12379,8 @@
         <v>9</v>
       </c>
       <c r="I214" s="1"/>
-      <c r="J214" s="71"/>
-      <c r="K214" s="73"/>
+      <c r="J214" s="62"/>
+      <c r="K214" s="64"/>
       <c r="L214" s="41" t="s">
         <v>53</v>
       </c>
@@ -12789,7 +12789,7 @@
       </c>
     </row>
     <row r="221" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A221" s="62">
+      <c r="A221" s="68">
         <v>6</v>
       </c>
       <c r="B221" s="34" t="s">
@@ -12814,7 +12814,7 @@
         <v>105.9126037429357</v>
       </c>
       <c r="I221" s="4"/>
-      <c r="J221" s="62">
+      <c r="J221" s="68">
         <v>6</v>
       </c>
       <c r="K221" s="34" t="s">
@@ -12854,7 +12854,7 @@
       </c>
     </row>
     <row r="222" spans="1:23" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A222" s="63"/>
+      <c r="A222" s="69"/>
       <c r="B222" s="35" t="s">
         <v>16</v>
       </c>
@@ -12877,7 +12877,7 @@
         <v>99.512296708627545</v>
       </c>
       <c r="I222" s="4"/>
-      <c r="J222" s="63"/>
+      <c r="J222" s="69"/>
       <c r="K222" s="35" t="s">
         <v>16</v>
       </c>
@@ -12915,7 +12915,7 @@
       </c>
     </row>
     <row r="223" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A223" s="62">
+      <c r="A223" s="68">
         <v>7</v>
       </c>
       <c r="B223" s="32" t="s">
@@ -12940,7 +12940,7 @@
         <v>102.67201902828714</v>
       </c>
       <c r="I223" s="4"/>
-      <c r="J223" s="62">
+      <c r="J223" s="68">
         <v>7</v>
       </c>
       <c r="K223" s="32" t="s">
@@ -12980,7 +12980,7 @@
       </c>
     </row>
     <row r="224" spans="1:23" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A224" s="64"/>
+      <c r="A224" s="70"/>
       <c r="B224" s="36" t="s">
         <v>18</v>
       </c>
@@ -13003,7 +13003,7 @@
         <v>109.7308790193191</v>
       </c>
       <c r="I224" s="4"/>
-      <c r="J224" s="64"/>
+      <c r="J224" s="70"/>
       <c r="K224" s="36" t="s">
         <v>18</v>
       </c>
@@ -13041,10 +13041,10 @@
       </c>
     </row>
     <row r="225" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A225" s="65" t="s">
+      <c r="A225" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="B225" s="66"/>
+      <c r="B225" s="72"/>
       <c r="C225" s="17">
         <v>2775.3961999999997</v>
       </c>
@@ -13064,10 +13064,10 @@
         <v>99.630474380558738</v>
       </c>
       <c r="I225" s="4"/>
-      <c r="J225" s="65" t="s">
+      <c r="J225" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="K225" s="66"/>
+      <c r="K225" s="72"/>
       <c r="L225" s="17">
         <v>2775.3961999999997</v>
       </c>
@@ -13168,146 +13168,94 @@
     </row>
   </sheetData>
   <mergeCells count="252">
-    <mergeCell ref="A94:H94"/>
-    <mergeCell ref="A95:C95"/>
-    <mergeCell ref="A77:H77"/>
-    <mergeCell ref="A78:B78"/>
-    <mergeCell ref="A79:A81"/>
-    <mergeCell ref="B79:B81"/>
-    <mergeCell ref="C79:H79"/>
-    <mergeCell ref="A88:A89"/>
-    <mergeCell ref="A90:A91"/>
-    <mergeCell ref="A92:B92"/>
-    <mergeCell ref="J92:K92"/>
-    <mergeCell ref="C80:D80"/>
-    <mergeCell ref="J79:J81"/>
-    <mergeCell ref="K79:K81"/>
-    <mergeCell ref="J88:J89"/>
-    <mergeCell ref="J90:J91"/>
-    <mergeCell ref="L79:Q79"/>
-    <mergeCell ref="L80:M80"/>
-    <mergeCell ref="N80:O80"/>
-    <mergeCell ref="P80:Q80"/>
-    <mergeCell ref="E80:F80"/>
-    <mergeCell ref="G80:H80"/>
-    <mergeCell ref="A115:H115"/>
-    <mergeCell ref="A116:B116"/>
-    <mergeCell ref="A117:A119"/>
-    <mergeCell ref="B117:B119"/>
-    <mergeCell ref="C117:H117"/>
-    <mergeCell ref="J117:J119"/>
-    <mergeCell ref="K117:K119"/>
-    <mergeCell ref="L117:Q117"/>
-    <mergeCell ref="C118:D118"/>
-    <mergeCell ref="E118:F118"/>
-    <mergeCell ref="G118:H118"/>
-    <mergeCell ref="L118:M118"/>
-    <mergeCell ref="N118:O118"/>
-    <mergeCell ref="P118:Q118"/>
-    <mergeCell ref="A126:A127"/>
-    <mergeCell ref="J126:J127"/>
-    <mergeCell ref="A128:A129"/>
-    <mergeCell ref="J128:J129"/>
-    <mergeCell ref="A130:B130"/>
-    <mergeCell ref="J130:K130"/>
-    <mergeCell ref="A132:H132"/>
-    <mergeCell ref="A134:H134"/>
-    <mergeCell ref="A135:B135"/>
-    <mergeCell ref="A136:A138"/>
-    <mergeCell ref="B136:B138"/>
-    <mergeCell ref="C136:H136"/>
-    <mergeCell ref="J136:J138"/>
-    <mergeCell ref="K136:K138"/>
-    <mergeCell ref="L136:Q136"/>
-    <mergeCell ref="C137:D137"/>
-    <mergeCell ref="E137:F137"/>
-    <mergeCell ref="G137:H137"/>
-    <mergeCell ref="L137:M137"/>
-    <mergeCell ref="N137:O137"/>
-    <mergeCell ref="P137:Q137"/>
-    <mergeCell ref="A145:A146"/>
-    <mergeCell ref="J145:J146"/>
-    <mergeCell ref="A147:A148"/>
-    <mergeCell ref="J147:J148"/>
-    <mergeCell ref="A149:B149"/>
-    <mergeCell ref="J149:K149"/>
-    <mergeCell ref="A151:H151"/>
-    <mergeCell ref="A153:H153"/>
-    <mergeCell ref="A154:B154"/>
-    <mergeCell ref="A155:A157"/>
-    <mergeCell ref="B155:B157"/>
-    <mergeCell ref="C155:H155"/>
-    <mergeCell ref="J155:J157"/>
-    <mergeCell ref="K155:K157"/>
-    <mergeCell ref="L155:Q155"/>
-    <mergeCell ref="C156:D156"/>
-    <mergeCell ref="E156:F156"/>
-    <mergeCell ref="G156:H156"/>
-    <mergeCell ref="L156:M156"/>
-    <mergeCell ref="N156:O156"/>
-    <mergeCell ref="P156:Q156"/>
-    <mergeCell ref="A164:A165"/>
-    <mergeCell ref="J164:J165"/>
-    <mergeCell ref="A166:A167"/>
-    <mergeCell ref="J166:J167"/>
-    <mergeCell ref="A168:B168"/>
-    <mergeCell ref="J168:K168"/>
-    <mergeCell ref="A170:H170"/>
-    <mergeCell ref="A172:H172"/>
-    <mergeCell ref="A173:B173"/>
-    <mergeCell ref="A174:A176"/>
-    <mergeCell ref="B174:B176"/>
-    <mergeCell ref="C174:H174"/>
-    <mergeCell ref="J174:J176"/>
-    <mergeCell ref="K174:K176"/>
-    <mergeCell ref="L174:Q174"/>
-    <mergeCell ref="C175:D175"/>
-    <mergeCell ref="E175:F175"/>
-    <mergeCell ref="G175:H175"/>
-    <mergeCell ref="L175:M175"/>
-    <mergeCell ref="N175:O175"/>
-    <mergeCell ref="P175:Q175"/>
-    <mergeCell ref="A183:A184"/>
-    <mergeCell ref="J183:J184"/>
-    <mergeCell ref="A185:A186"/>
-    <mergeCell ref="J185:J186"/>
-    <mergeCell ref="A187:B187"/>
-    <mergeCell ref="J187:K187"/>
-    <mergeCell ref="A189:H189"/>
-    <mergeCell ref="A191:H191"/>
-    <mergeCell ref="A192:B192"/>
-    <mergeCell ref="A193:A195"/>
-    <mergeCell ref="B193:B195"/>
-    <mergeCell ref="C193:H193"/>
-    <mergeCell ref="J193:J195"/>
-    <mergeCell ref="K193:K195"/>
-    <mergeCell ref="L193:Q193"/>
-    <mergeCell ref="C194:D194"/>
-    <mergeCell ref="E194:F194"/>
-    <mergeCell ref="G194:H194"/>
-    <mergeCell ref="L194:M194"/>
-    <mergeCell ref="N194:O194"/>
-    <mergeCell ref="P194:Q194"/>
-    <mergeCell ref="A202:A203"/>
-    <mergeCell ref="J202:J203"/>
-    <mergeCell ref="A204:A205"/>
-    <mergeCell ref="J204:J205"/>
-    <mergeCell ref="A206:B206"/>
-    <mergeCell ref="J206:K206"/>
-    <mergeCell ref="A208:H208"/>
-    <mergeCell ref="A210:H210"/>
-    <mergeCell ref="A211:B211"/>
-    <mergeCell ref="A212:A214"/>
-    <mergeCell ref="B212:B214"/>
-    <mergeCell ref="C212:H212"/>
-    <mergeCell ref="K212:K214"/>
-    <mergeCell ref="L212:Q212"/>
-    <mergeCell ref="C213:D213"/>
-    <mergeCell ref="E213:F213"/>
-    <mergeCell ref="G213:H213"/>
-    <mergeCell ref="L213:M213"/>
-    <mergeCell ref="N213:O213"/>
-    <mergeCell ref="P213:Q213"/>
+    <mergeCell ref="L3:Q3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="J12:J13"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="A73:B73"/>
+    <mergeCell ref="J73:K73"/>
+    <mergeCell ref="A75:H75"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="C3:H3"/>
+    <mergeCell ref="J3:J5"/>
+    <mergeCell ref="K3:K5"/>
+    <mergeCell ref="J50:J51"/>
+    <mergeCell ref="A52:A53"/>
+    <mergeCell ref="J52:J53"/>
+    <mergeCell ref="A54:B54"/>
+    <mergeCell ref="J54:K54"/>
+    <mergeCell ref="A56:H56"/>
+    <mergeCell ref="A50:A51"/>
+    <mergeCell ref="K60:K62"/>
+    <mergeCell ref="A41:A43"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="C41:H41"/>
+    <mergeCell ref="J41:J43"/>
+    <mergeCell ref="K41:K43"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="L60:Q60"/>
+    <mergeCell ref="C61:D61"/>
+    <mergeCell ref="E61:F61"/>
+    <mergeCell ref="G61:H61"/>
+    <mergeCell ref="L61:M61"/>
+    <mergeCell ref="N61:O61"/>
+    <mergeCell ref="P61:Q61"/>
+    <mergeCell ref="A60:A62"/>
+    <mergeCell ref="B60:B62"/>
+    <mergeCell ref="C60:H60"/>
+    <mergeCell ref="J60:J62"/>
+    <mergeCell ref="L41:Q41"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="L42:M42"/>
+    <mergeCell ref="N42:O42"/>
+    <mergeCell ref="P42:Q42"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="J35:K35"/>
+    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="J22:J24"/>
+    <mergeCell ref="K22:K24"/>
+    <mergeCell ref="L22:Q22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="L23:M23"/>
+    <mergeCell ref="N23:O23"/>
+    <mergeCell ref="P23:Q23"/>
+    <mergeCell ref="L98:Q98"/>
+    <mergeCell ref="C99:D99"/>
+    <mergeCell ref="E99:F99"/>
+    <mergeCell ref="G99:H99"/>
+    <mergeCell ref="L99:M99"/>
+    <mergeCell ref="N99:O99"/>
+    <mergeCell ref="P99:Q99"/>
+    <mergeCell ref="J107:J108"/>
+    <mergeCell ref="A109:A110"/>
+    <mergeCell ref="J109:J110"/>
     <mergeCell ref="A58:H58"/>
     <mergeCell ref="A59:B59"/>
     <mergeCell ref="A221:A222"/>
@@ -13332,94 +13280,146 @@
     <mergeCell ref="J69:J70"/>
     <mergeCell ref="A71:A72"/>
     <mergeCell ref="J71:J72"/>
-    <mergeCell ref="L98:Q98"/>
-    <mergeCell ref="C99:D99"/>
-    <mergeCell ref="E99:F99"/>
-    <mergeCell ref="G99:H99"/>
-    <mergeCell ref="L99:M99"/>
-    <mergeCell ref="N99:O99"/>
-    <mergeCell ref="P99:Q99"/>
-    <mergeCell ref="J107:J108"/>
-    <mergeCell ref="A109:A110"/>
-    <mergeCell ref="J109:J110"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:A24"/>
-    <mergeCell ref="B22:B24"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="J22:J24"/>
-    <mergeCell ref="K22:K24"/>
-    <mergeCell ref="L22:Q22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="G23:H23"/>
-    <mergeCell ref="L23:M23"/>
-    <mergeCell ref="N23:O23"/>
-    <mergeCell ref="P23:Q23"/>
-    <mergeCell ref="L41:Q41"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="L42:M42"/>
-    <mergeCell ref="N42:O42"/>
-    <mergeCell ref="P42:Q42"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="J35:K35"/>
-    <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A39:H39"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="L60:Q60"/>
-    <mergeCell ref="C61:D61"/>
-    <mergeCell ref="E61:F61"/>
-    <mergeCell ref="G61:H61"/>
-    <mergeCell ref="L61:M61"/>
-    <mergeCell ref="N61:O61"/>
-    <mergeCell ref="P61:Q61"/>
-    <mergeCell ref="A60:A62"/>
-    <mergeCell ref="B60:B62"/>
-    <mergeCell ref="C60:H60"/>
-    <mergeCell ref="J60:J62"/>
-    <mergeCell ref="A73:B73"/>
-    <mergeCell ref="J73:K73"/>
-    <mergeCell ref="A75:H75"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:A5"/>
-    <mergeCell ref="B3:B5"/>
-    <mergeCell ref="C3:H3"/>
-    <mergeCell ref="J3:J5"/>
-    <mergeCell ref="K3:K5"/>
-    <mergeCell ref="J50:J51"/>
-    <mergeCell ref="A52:A53"/>
-    <mergeCell ref="J52:J53"/>
-    <mergeCell ref="A54:B54"/>
-    <mergeCell ref="J54:K54"/>
-    <mergeCell ref="A56:H56"/>
-    <mergeCell ref="A50:A51"/>
-    <mergeCell ref="K60:K62"/>
-    <mergeCell ref="A41:A43"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="C41:H41"/>
-    <mergeCell ref="J41:J43"/>
-    <mergeCell ref="K41:K43"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="L3:Q3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="N4:O4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="A18:H18"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="J12:J13"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="J14:J15"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="A212:A214"/>
+    <mergeCell ref="B212:B214"/>
+    <mergeCell ref="C212:H212"/>
+    <mergeCell ref="K212:K214"/>
+    <mergeCell ref="L212:Q212"/>
+    <mergeCell ref="C213:D213"/>
+    <mergeCell ref="E213:F213"/>
+    <mergeCell ref="G213:H213"/>
+    <mergeCell ref="L213:M213"/>
+    <mergeCell ref="N213:O213"/>
+    <mergeCell ref="P213:Q213"/>
+    <mergeCell ref="A202:A203"/>
+    <mergeCell ref="J202:J203"/>
+    <mergeCell ref="A204:A205"/>
+    <mergeCell ref="J204:J205"/>
+    <mergeCell ref="A206:B206"/>
+    <mergeCell ref="J206:K206"/>
+    <mergeCell ref="A208:H208"/>
+    <mergeCell ref="A210:H210"/>
+    <mergeCell ref="A211:B211"/>
+    <mergeCell ref="A193:A195"/>
+    <mergeCell ref="B193:B195"/>
+    <mergeCell ref="C193:H193"/>
+    <mergeCell ref="J193:J195"/>
+    <mergeCell ref="K193:K195"/>
+    <mergeCell ref="L193:Q193"/>
+    <mergeCell ref="C194:D194"/>
+    <mergeCell ref="E194:F194"/>
+    <mergeCell ref="G194:H194"/>
+    <mergeCell ref="L194:M194"/>
+    <mergeCell ref="N194:O194"/>
+    <mergeCell ref="P194:Q194"/>
+    <mergeCell ref="A183:A184"/>
+    <mergeCell ref="J183:J184"/>
+    <mergeCell ref="A185:A186"/>
+    <mergeCell ref="J185:J186"/>
+    <mergeCell ref="A187:B187"/>
+    <mergeCell ref="J187:K187"/>
+    <mergeCell ref="A189:H189"/>
+    <mergeCell ref="A191:H191"/>
+    <mergeCell ref="A192:B192"/>
+    <mergeCell ref="A174:A176"/>
+    <mergeCell ref="B174:B176"/>
+    <mergeCell ref="C174:H174"/>
+    <mergeCell ref="J174:J176"/>
+    <mergeCell ref="K174:K176"/>
+    <mergeCell ref="L174:Q174"/>
+    <mergeCell ref="C175:D175"/>
+    <mergeCell ref="E175:F175"/>
+    <mergeCell ref="G175:H175"/>
+    <mergeCell ref="L175:M175"/>
+    <mergeCell ref="N175:O175"/>
+    <mergeCell ref="P175:Q175"/>
+    <mergeCell ref="A164:A165"/>
+    <mergeCell ref="J164:J165"/>
+    <mergeCell ref="A166:A167"/>
+    <mergeCell ref="J166:J167"/>
+    <mergeCell ref="A168:B168"/>
+    <mergeCell ref="J168:K168"/>
+    <mergeCell ref="A170:H170"/>
+    <mergeCell ref="A172:H172"/>
+    <mergeCell ref="A173:B173"/>
+    <mergeCell ref="A155:A157"/>
+    <mergeCell ref="B155:B157"/>
+    <mergeCell ref="C155:H155"/>
+    <mergeCell ref="J155:J157"/>
+    <mergeCell ref="K155:K157"/>
+    <mergeCell ref="L155:Q155"/>
+    <mergeCell ref="C156:D156"/>
+    <mergeCell ref="E156:F156"/>
+    <mergeCell ref="G156:H156"/>
+    <mergeCell ref="L156:M156"/>
+    <mergeCell ref="N156:O156"/>
+    <mergeCell ref="P156:Q156"/>
+    <mergeCell ref="A145:A146"/>
+    <mergeCell ref="J145:J146"/>
+    <mergeCell ref="A147:A148"/>
+    <mergeCell ref="J147:J148"/>
+    <mergeCell ref="A149:B149"/>
+    <mergeCell ref="J149:K149"/>
+    <mergeCell ref="A151:H151"/>
+    <mergeCell ref="A153:H153"/>
+    <mergeCell ref="A154:B154"/>
+    <mergeCell ref="A136:A138"/>
+    <mergeCell ref="B136:B138"/>
+    <mergeCell ref="C136:H136"/>
+    <mergeCell ref="J136:J138"/>
+    <mergeCell ref="K136:K138"/>
+    <mergeCell ref="L136:Q136"/>
+    <mergeCell ref="C137:D137"/>
+    <mergeCell ref="E137:F137"/>
+    <mergeCell ref="G137:H137"/>
+    <mergeCell ref="L137:M137"/>
+    <mergeCell ref="N137:O137"/>
+    <mergeCell ref="P137:Q137"/>
+    <mergeCell ref="A126:A127"/>
+    <mergeCell ref="J126:J127"/>
+    <mergeCell ref="A128:A129"/>
+    <mergeCell ref="J128:J129"/>
+    <mergeCell ref="A130:B130"/>
+    <mergeCell ref="J130:K130"/>
+    <mergeCell ref="A132:H132"/>
+    <mergeCell ref="A134:H134"/>
+    <mergeCell ref="A135:B135"/>
+    <mergeCell ref="A115:H115"/>
+    <mergeCell ref="A116:B116"/>
+    <mergeCell ref="A117:A119"/>
+    <mergeCell ref="B117:B119"/>
+    <mergeCell ref="C117:H117"/>
+    <mergeCell ref="J117:J119"/>
+    <mergeCell ref="K117:K119"/>
+    <mergeCell ref="L117:Q117"/>
+    <mergeCell ref="C118:D118"/>
+    <mergeCell ref="E118:F118"/>
+    <mergeCell ref="G118:H118"/>
+    <mergeCell ref="L118:M118"/>
+    <mergeCell ref="N118:O118"/>
+    <mergeCell ref="P118:Q118"/>
+    <mergeCell ref="J92:K92"/>
+    <mergeCell ref="C80:D80"/>
+    <mergeCell ref="J79:J81"/>
+    <mergeCell ref="K79:K81"/>
+    <mergeCell ref="J88:J89"/>
+    <mergeCell ref="J90:J91"/>
+    <mergeCell ref="L79:Q79"/>
+    <mergeCell ref="L80:M80"/>
+    <mergeCell ref="N80:O80"/>
+    <mergeCell ref="P80:Q80"/>
+    <mergeCell ref="E80:F80"/>
+    <mergeCell ref="G80:H80"/>
+    <mergeCell ref="A94:H94"/>
+    <mergeCell ref="A95:C95"/>
+    <mergeCell ref="A77:H77"/>
+    <mergeCell ref="A78:B78"/>
+    <mergeCell ref="A79:A81"/>
+    <mergeCell ref="B79:B81"/>
+    <mergeCell ref="C79:H79"/>
+    <mergeCell ref="A88:A89"/>
+    <mergeCell ref="A90:A91"/>
+    <mergeCell ref="A92:B92"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>